<commit_message>
Fix manual transcription error and WER calcualtion. Filip reviewed my work by also listening to the video and he found a few things that I missheard. I corrected those in the transcript and I recalculated the WER rates for both models. However, since there only were a few changes made to my transcribtion, the changes didn't make much of a difference.
</commit_message>
<xml_diff>
--- a/deliverables/Task 2/STT_AssemblyAI.xlsx
+++ b/deliverables/Task 2/STT_AssemblyAI.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\rzvn1\Documents\fae2-nlpr-group-group-12-1\deliverables\Task 2\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{4FC42535-6962-487D-8B6D-95659D712DC5}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{D875D6CD-E4E8-49AA-8203-87D8A32E16C0}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12456" xr2:uid="{48823F93-F958-48E2-9AF7-7396F4F03D9F}"/>
   </bookViews>
@@ -33,7 +33,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="1400" uniqueCount="1015">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="1400" uniqueCount="1016">
   <si>
     <t>And in 2010, it was bought by the Leyva family.</t>
   </si>
@@ -1754,9 +1754,6 @@
     <t>Okay.</t>
   </si>
   <si>
-    <t>I took the collateral, you know, the house.</t>
-  </si>
-  <si>
     <t>Wow!</t>
   </si>
   <si>
@@ -3071,13 +3068,19 @@
     <t>Dough ball, wet, soggy, horrible dough.</t>
   </si>
   <si>
-    <t>TOTAL: 75</t>
-  </si>
-  <si>
     <t>N = 1223 Words</t>
   </si>
   <si>
-    <t>WER: 75/1264 = 0.05933/5.933%</t>
+    <t>I took the collateral, you know, the house, and her house.</t>
+  </si>
+  <si>
+    <t>What is gonna bring the people in?</t>
+  </si>
+  <si>
+    <t>TOTAL: 74</t>
+  </si>
+  <si>
+    <t>WER: 74/1262 = 0.05863/5.863%</t>
   </si>
 </sst>
 </file>
@@ -4042,10 +4045,10 @@
   <sheetData>
     <row r="1" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A1" t="s">
-        <v>989</v>
+        <v>988</v>
       </c>
       <c r="B1" t="s">
-        <v>575</v>
+        <v>574</v>
       </c>
       <c r="C1" s="1" t="s">
         <v>499</v>
@@ -4057,23 +4060,23 @@
         <v>500</v>
       </c>
       <c r="F1" t="s">
-        <v>1013</v>
+        <v>1011</v>
       </c>
     </row>
     <row r="2" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A2" t="s">
-        <v>578</v>
+        <v>577</v>
       </c>
       <c r="B2" t="s">
-        <v>990</v>
+        <v>989</v>
       </c>
     </row>
     <row r="3" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A3" t="s">
-        <v>579</v>
+        <v>578</v>
       </c>
       <c r="B3" t="s">
-        <v>579</v>
+        <v>578</v>
       </c>
     </row>
     <row r="4" spans="1:6" x14ac:dyDescent="0.3">
@@ -4102,34 +4105,34 @@
     </row>
     <row r="7" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A7" t="s">
-        <v>580</v>
+        <v>579</v>
       </c>
       <c r="B7" t="s">
-        <v>580</v>
+        <v>579</v>
       </c>
     </row>
     <row r="8" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A8" t="s">
-        <v>581</v>
+        <v>580</v>
       </c>
       <c r="B8" t="s">
-        <v>581</v>
+        <v>580</v>
       </c>
     </row>
     <row r="9" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A9" t="s">
-        <v>582</v>
+        <v>581</v>
       </c>
       <c r="B9" t="s">
-        <v>582</v>
+        <v>581</v>
       </c>
     </row>
     <row r="10" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A10" s="1" t="s">
-        <v>583</v>
+        <v>582</v>
       </c>
       <c r="B10" s="1" t="s">
-        <v>991</v>
+        <v>990</v>
       </c>
       <c r="C10">
         <v>1</v>
@@ -4169,10 +4172,10 @@
     </row>
     <row r="15" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A15" s="3" t="s">
-        <v>584</v>
+        <v>583</v>
       </c>
       <c r="B15" s="3" t="s">
-        <v>992</v>
+        <v>991</v>
       </c>
       <c r="E15">
         <v>1</v>
@@ -4204,18 +4207,21 @@
     </row>
     <row r="19" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A19" t="s">
-        <v>585</v>
+        <v>584</v>
       </c>
       <c r="B19" t="s">
-        <v>585</v>
+        <v>584</v>
       </c>
     </row>
     <row r="20" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A20" t="s">
-        <v>586</v>
+        <v>585</v>
       </c>
       <c r="B20" t="s">
-        <v>586</v>
+        <v>1013</v>
+      </c>
+      <c r="C20">
+        <v>1</v>
       </c>
     </row>
     <row r="21" spans="1:5" x14ac:dyDescent="0.3">
@@ -4244,18 +4250,18 @@
     </row>
     <row r="24" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A24" t="s">
-        <v>587</v>
+        <v>586</v>
       </c>
       <c r="B24" t="s">
-        <v>587</v>
+        <v>586</v>
       </c>
     </row>
     <row r="25" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A25" s="2" t="s">
-        <v>588</v>
+        <v>587</v>
       </c>
       <c r="B25" s="2" t="s">
-        <v>993</v>
+        <v>992</v>
       </c>
       <c r="D25">
         <v>5</v>
@@ -4266,26 +4272,26 @@
     </row>
     <row r="26" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A26" t="s">
-        <v>589</v>
+        <v>588</v>
       </c>
       <c r="B26" t="s">
-        <v>994</v>
+        <v>993</v>
       </c>
     </row>
     <row r="27" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A27" t="s">
-        <v>590</v>
+        <v>589</v>
       </c>
       <c r="B27" t="s">
-        <v>590</v>
+        <v>589</v>
       </c>
     </row>
     <row r="28" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A28" t="s">
-        <v>591</v>
+        <v>590</v>
       </c>
       <c r="B28" t="s">
-        <v>591</v>
+        <v>590</v>
       </c>
     </row>
     <row r="29" spans="1:5" x14ac:dyDescent="0.3">
@@ -4298,10 +4304,10 @@
     </row>
     <row r="30" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A30" t="s">
-        <v>592</v>
+        <v>591</v>
       </c>
       <c r="B30" t="s">
-        <v>592</v>
+        <v>591</v>
       </c>
     </row>
     <row r="31" spans="1:5" x14ac:dyDescent="0.3">
@@ -4338,7 +4344,7 @@
     </row>
     <row r="35" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A35" s="1" t="s">
-        <v>593</v>
+        <v>592</v>
       </c>
       <c r="B35" s="1" t="s">
         <v>18</v>
@@ -4374,7 +4380,7 @@
     </row>
     <row r="39" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A39" t="s">
-        <v>594</v>
+        <v>593</v>
       </c>
       <c r="B39" t="s">
         <v>21</v>
@@ -4411,7 +4417,7 @@
     </row>
     <row r="44" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A44" s="3" t="s">
-        <v>595</v>
+        <v>594</v>
       </c>
       <c r="B44" s="3" t="s">
         <v>503</v>
@@ -4430,18 +4436,18 @@
     </row>
     <row r="46" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A46" t="s">
-        <v>596</v>
+        <v>595</v>
       </c>
       <c r="B46" t="s">
-        <v>596</v>
+        <v>595</v>
       </c>
     </row>
     <row r="47" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A47" t="s">
-        <v>597</v>
+        <v>596</v>
       </c>
       <c r="B47" t="s">
-        <v>597</v>
+        <v>596</v>
       </c>
     </row>
     <row r="48" spans="1:5" x14ac:dyDescent="0.3">
@@ -4462,7 +4468,7 @@
     </row>
     <row r="50" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A50" s="1" t="s">
-        <v>598</v>
+        <v>597</v>
       </c>
       <c r="B50" s="1" t="s">
         <v>567</v>
@@ -4473,18 +4479,18 @@
     </row>
     <row r="51" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A51" t="s">
-        <v>599</v>
+        <v>598</v>
       </c>
       <c r="B51" t="s">
-        <v>599</v>
+        <v>598</v>
       </c>
     </row>
     <row r="52" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A52" t="s">
-        <v>600</v>
+        <v>599</v>
       </c>
       <c r="B52" t="s">
-        <v>600</v>
+        <v>599</v>
       </c>
     </row>
     <row r="53" spans="1:3" x14ac:dyDescent="0.3">
@@ -4505,10 +4511,10 @@
     </row>
     <row r="55" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A55" t="s">
-        <v>601</v>
+        <v>600</v>
       </c>
       <c r="B55" t="s">
-        <v>601</v>
+        <v>600</v>
       </c>
     </row>
     <row r="56" spans="1:3" x14ac:dyDescent="0.3">
@@ -4529,34 +4535,34 @@
     </row>
     <row r="58" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A58" t="s">
-        <v>602</v>
+        <v>601</v>
       </c>
       <c r="B58" t="s">
-        <v>602</v>
+        <v>601</v>
       </c>
     </row>
     <row r="59" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A59" t="s">
-        <v>603</v>
+        <v>602</v>
       </c>
       <c r="B59" t="s">
-        <v>603</v>
+        <v>602</v>
       </c>
     </row>
     <row r="60" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A60" t="s">
-        <v>604</v>
+        <v>603</v>
       </c>
       <c r="B60" t="s">
-        <v>604</v>
+        <v>603</v>
       </c>
     </row>
     <row r="61" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A61" t="s">
-        <v>605</v>
+        <v>604</v>
       </c>
       <c r="B61" t="s">
-        <v>605</v>
+        <v>604</v>
       </c>
     </row>
     <row r="62" spans="1:3" x14ac:dyDescent="0.3">
@@ -4569,10 +4575,10 @@
     </row>
     <row r="63" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A63" t="s">
-        <v>606</v>
+        <v>605</v>
       </c>
       <c r="B63" t="s">
-        <v>606</v>
+        <v>605</v>
       </c>
     </row>
     <row r="64" spans="1:3" x14ac:dyDescent="0.3">
@@ -4626,10 +4632,10 @@
     </row>
     <row r="70" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A70" t="s">
-        <v>607</v>
+        <v>606</v>
       </c>
       <c r="B70" t="s">
-        <v>607</v>
+        <v>606</v>
       </c>
     </row>
     <row r="71" spans="1:5" x14ac:dyDescent="0.3">
@@ -4698,10 +4704,10 @@
     </row>
     <row r="79" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A79" t="s">
-        <v>608</v>
+        <v>607</v>
       </c>
       <c r="B79" t="s">
-        <v>608</v>
+        <v>607</v>
       </c>
     </row>
     <row r="80" spans="1:5" x14ac:dyDescent="0.3">
@@ -4714,10 +4720,10 @@
     </row>
     <row r="81" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A81" t="s">
-        <v>609</v>
+        <v>608</v>
       </c>
       <c r="B81" t="s">
-        <v>609</v>
+        <v>608</v>
       </c>
     </row>
     <row r="82" spans="1:5" x14ac:dyDescent="0.3">
@@ -4754,10 +4760,10 @@
     </row>
     <row r="86" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A86" s="1" t="s">
-        <v>610</v>
+        <v>609</v>
       </c>
       <c r="B86" s="1" t="s">
-        <v>995</v>
+        <v>994</v>
       </c>
       <c r="C86">
         <v>2</v>
@@ -4765,10 +4771,10 @@
     </row>
     <row r="87" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A87" s="2" t="s">
-        <v>611</v>
+        <v>610</v>
       </c>
       <c r="B87" s="2" t="s">
-        <v>996</v>
+        <v>995</v>
       </c>
       <c r="D87">
         <v>2</v>
@@ -4792,7 +4798,7 @@
     </row>
     <row r="90" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A90" t="s">
-        <v>612</v>
+        <v>611</v>
       </c>
       <c r="B90" s="3" t="s">
         <v>50</v>
@@ -4827,10 +4833,10 @@
     </row>
     <row r="94" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A94" s="3" t="s">
-        <v>613</v>
+        <v>612</v>
       </c>
       <c r="B94" s="3" t="s">
-        <v>997</v>
+        <v>996</v>
       </c>
       <c r="E94">
         <v>1</v>
@@ -4838,10 +4844,10 @@
     </row>
     <row r="95" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A95" s="3" t="s">
-        <v>614</v>
+        <v>613</v>
       </c>
       <c r="B95" s="3" t="s">
-        <v>998</v>
+        <v>997</v>
       </c>
       <c r="E95">
         <v>2</v>
@@ -4849,10 +4855,10 @@
     </row>
     <row r="96" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A96" s="1" t="s">
-        <v>615</v>
+        <v>614</v>
       </c>
       <c r="B96" s="1" t="s">
-        <v>999</v>
+        <v>998</v>
       </c>
       <c r="C96">
         <v>1</v>
@@ -4860,7 +4866,7 @@
     </row>
     <row r="97" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A97" s="3" t="s">
-        <v>616</v>
+        <v>615</v>
       </c>
       <c r="B97" s="3" t="s">
         <v>506</v>
@@ -4868,7 +4874,7 @@
     </row>
     <row r="98" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A98" s="3" t="s">
-        <v>617</v>
+        <v>616</v>
       </c>
       <c r="B98" s="3"/>
       <c r="E98">
@@ -4918,7 +4924,7 @@
     </row>
     <row r="104" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A104" t="s">
-        <v>618</v>
+        <v>617</v>
       </c>
       <c r="B104" t="s">
         <v>571</v>
@@ -4942,10 +4948,10 @@
     </row>
     <row r="107" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A107" t="s">
-        <v>619</v>
+        <v>618</v>
       </c>
       <c r="B107" t="s">
-        <v>619</v>
+        <v>618</v>
       </c>
     </row>
     <row r="108" spans="1:5" x14ac:dyDescent="0.3">
@@ -4958,10 +4964,10 @@
     </row>
     <row r="109" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A109" s="3" t="s">
-        <v>620</v>
+        <v>619</v>
       </c>
       <c r="B109" s="3" t="s">
-        <v>1000</v>
+        <v>999</v>
       </c>
       <c r="D109">
         <v>1</v>
@@ -4972,7 +4978,7 @@
     </row>
     <row r="110" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A110" t="s">
-        <v>621</v>
+        <v>620</v>
       </c>
     </row>
     <row r="111" spans="1:5" x14ac:dyDescent="0.3">
@@ -5018,21 +5024,21 @@
     </row>
     <row r="116" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A116" s="3" t="s">
-        <v>622</v>
+        <v>621</v>
       </c>
       <c r="B116" s="3" t="s">
-        <v>573</v>
+        <v>1012</v>
       </c>
       <c r="D116">
         <v>3</v>
       </c>
       <c r="E116">
-        <v>4</v>
+        <v>2</v>
       </c>
     </row>
     <row r="117" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A117" s="3" t="s">
-        <v>623</v>
+        <v>622</v>
       </c>
       <c r="B117" s="3" t="s">
         <v>507</v>
@@ -5043,16 +5049,16 @@
     </row>
     <row r="118" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A118" t="s">
-        <v>624</v>
+        <v>623</v>
       </c>
       <c r="B118" t="s">
-        <v>624</v>
+        <v>623</v>
       </c>
     </row>
     <row r="119" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A119" s="3"/>
       <c r="B119" s="3" t="s">
-        <v>574</v>
+        <v>573</v>
       </c>
       <c r="E119">
         <v>1</v>
@@ -5068,10 +5074,10 @@
     </row>
     <row r="121" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A121" t="s">
-        <v>625</v>
+        <v>624</v>
       </c>
       <c r="B121" t="s">
-        <v>625</v>
+        <v>624</v>
       </c>
     </row>
     <row r="122" spans="1:5" x14ac:dyDescent="0.3">
@@ -5109,7 +5115,7 @@
     </row>
     <row r="126" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A126" t="s">
-        <v>626</v>
+        <v>625</v>
       </c>
       <c r="B126" t="s">
         <v>66</v>
@@ -5130,10 +5136,10 @@
     </row>
     <row r="129" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A129" t="s">
-        <v>627</v>
+        <v>626</v>
       </c>
       <c r="B129" t="s">
-        <v>627</v>
+        <v>626</v>
       </c>
     </row>
     <row r="130" spans="1:5" x14ac:dyDescent="0.3">
@@ -5147,7 +5153,7 @@
     <row r="131" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A131" s="3"/>
       <c r="B131" s="3" t="s">
-        <v>574</v>
+        <v>573</v>
       </c>
       <c r="E131">
         <v>1</v>
@@ -5171,16 +5177,16 @@
     </row>
     <row r="134" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A134" t="s">
-        <v>628</v>
+        <v>627</v>
       </c>
       <c r="B134" t="s">
-        <v>628</v>
+        <v>627</v>
       </c>
     </row>
     <row r="135" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A135" s="3"/>
       <c r="B135" s="3" t="s">
-        <v>574</v>
+        <v>573</v>
       </c>
     </row>
     <row r="136" spans="1:5" x14ac:dyDescent="0.3">
@@ -5201,18 +5207,18 @@
     </row>
     <row r="138" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A138" t="s">
-        <v>629</v>
+        <v>628</v>
       </c>
       <c r="B138" t="s">
-        <v>1001</v>
+        <v>1000</v>
       </c>
     </row>
     <row r="139" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A139" s="3" t="s">
-        <v>630</v>
+        <v>629</v>
       </c>
       <c r="B139" s="3" t="s">
-        <v>576</v>
+        <v>575</v>
       </c>
       <c r="E139">
         <v>2</v>
@@ -5244,10 +5250,10 @@
     </row>
     <row r="143" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A143" s="1" t="s">
-        <v>631</v>
+        <v>630</v>
       </c>
       <c r="B143" s="1" t="s">
-        <v>1002</v>
+        <v>1001</v>
       </c>
       <c r="E143">
         <v>1</v>
@@ -5264,7 +5270,7 @@
     <row r="145" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A145" s="3"/>
       <c r="B145" s="3" t="s">
-        <v>577</v>
+        <v>576</v>
       </c>
       <c r="E145">
         <v>1</v>
@@ -5304,10 +5310,10 @@
     </row>
     <row r="150" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A150" t="s">
-        <v>632</v>
+        <v>631</v>
       </c>
       <c r="B150" t="s">
-        <v>1003</v>
+        <v>1002</v>
       </c>
     </row>
     <row r="151" spans="1:5" x14ac:dyDescent="0.3">
@@ -5320,10 +5326,10 @@
     </row>
     <row r="152" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A152" s="3" t="s">
-        <v>633</v>
+        <v>632</v>
       </c>
       <c r="B152" s="3" t="s">
-        <v>1004</v>
+        <v>1003</v>
       </c>
       <c r="C152">
         <v>1</v>
@@ -5342,10 +5348,10 @@
     </row>
     <row r="154" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A154" t="s">
-        <v>634</v>
+        <v>633</v>
       </c>
       <c r="B154" t="s">
-        <v>634</v>
+        <v>633</v>
       </c>
     </row>
     <row r="155" spans="1:5" x14ac:dyDescent="0.3">
@@ -5374,7 +5380,7 @@
     </row>
     <row r="158" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A158" s="3" t="s">
-        <v>635</v>
+        <v>634</v>
       </c>
       <c r="B158" s="3" t="s">
         <v>80</v>
@@ -5385,7 +5391,7 @@
     </row>
     <row r="159" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A159" t="s">
-        <v>636</v>
+        <v>635</v>
       </c>
       <c r="B159" t="s">
         <v>81</v>
@@ -5394,7 +5400,7 @@
     <row r="160" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A160" s="3"/>
       <c r="B160" s="3" t="s">
-        <v>574</v>
+        <v>573</v>
       </c>
       <c r="E160">
         <v>1</v>
@@ -5419,26 +5425,26 @@
     </row>
     <row r="163" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A163" t="s">
-        <v>637</v>
+        <v>636</v>
       </c>
       <c r="B163" t="s">
-        <v>637</v>
+        <v>636</v>
       </c>
     </row>
     <row r="164" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A164" t="s">
-        <v>638</v>
+        <v>637</v>
       </c>
       <c r="B164" t="s">
-        <v>638</v>
+        <v>637</v>
       </c>
     </row>
     <row r="165" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A165" t="s">
-        <v>639</v>
+        <v>638</v>
       </c>
       <c r="B165" t="s">
-        <v>639</v>
+        <v>638</v>
       </c>
     </row>
     <row r="166" spans="1:5" x14ac:dyDescent="0.3">
@@ -5451,10 +5457,10 @@
     </row>
     <row r="167" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A167" t="s">
-        <v>640</v>
+        <v>639</v>
       </c>
       <c r="B167" t="s">
-        <v>640</v>
+        <v>639</v>
       </c>
     </row>
     <row r="168" spans="1:5" x14ac:dyDescent="0.3">
@@ -5475,7 +5481,7 @@
     </row>
     <row r="170" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A170" s="2" t="s">
-        <v>641</v>
+        <v>640</v>
       </c>
       <c r="B170" s="2"/>
       <c r="D170">
@@ -5484,10 +5490,10 @@
     </row>
     <row r="171" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A171" t="s">
-        <v>642</v>
+        <v>641</v>
       </c>
       <c r="B171" t="s">
-        <v>1005</v>
+        <v>1004</v>
       </c>
     </row>
     <row r="172" spans="1:5" x14ac:dyDescent="0.3">
@@ -5533,10 +5539,10 @@
     </row>
     <row r="177" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A177" t="s">
-        <v>643</v>
+        <v>642</v>
       </c>
       <c r="B177" t="s">
-        <v>643</v>
+        <v>642</v>
       </c>
     </row>
     <row r="178" spans="1:5" x14ac:dyDescent="0.3">
@@ -5549,10 +5555,10 @@
     </row>
     <row r="179" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A179" t="s">
-        <v>644</v>
+        <v>643</v>
       </c>
       <c r="B179" t="s">
-        <v>644</v>
+        <v>643</v>
       </c>
     </row>
     <row r="180" spans="1:5" x14ac:dyDescent="0.3">
@@ -5566,10 +5572,10 @@
     </row>
     <row r="181" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A181" t="s">
-        <v>645</v>
+        <v>644</v>
       </c>
       <c r="B181" t="s">
-        <v>645</v>
+        <v>644</v>
       </c>
     </row>
     <row r="182" spans="1:5" x14ac:dyDescent="0.3">
@@ -5583,7 +5589,7 @@
     </row>
     <row r="183" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A183" t="s">
-        <v>646</v>
+        <v>645</v>
       </c>
       <c r="B183" t="s">
         <v>90</v>
@@ -5591,7 +5597,7 @@
     </row>
     <row r="184" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A184" s="1" t="s">
-        <v>647</v>
+        <v>646</v>
       </c>
       <c r="B184" s="1" t="s">
         <v>91</v>
@@ -5600,7 +5606,7 @@
     <row r="185" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A185" s="3"/>
       <c r="B185" s="3" t="s">
-        <v>1006</v>
+        <v>1005</v>
       </c>
       <c r="E185">
         <v>4</v>
@@ -5609,7 +5615,7 @@
     <row r="186" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A186" s="3"/>
       <c r="B186" s="3" t="s">
-        <v>1007</v>
+        <v>1006</v>
       </c>
       <c r="E186">
         <v>1</v>
@@ -5652,7 +5658,7 @@
         <v>95</v>
       </c>
       <c r="B191" s="3" t="s">
-        <v>1008</v>
+        <v>1007</v>
       </c>
       <c r="E191">
         <v>1</v>
@@ -5717,23 +5723,23 @@
     </row>
     <row r="199" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A199" t="s">
-        <v>648</v>
+        <v>647</v>
       </c>
       <c r="B199" t="s">
-        <v>1011</v>
+        <v>1010</v>
       </c>
     </row>
     <row r="200" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A200" t="s">
-        <v>649</v>
+        <v>648</v>
       </c>
     </row>
     <row r="201" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A201" s="1" t="s">
-        <v>650</v>
+        <v>649</v>
       </c>
       <c r="B201" s="1" t="s">
-        <v>1009</v>
+        <v>1008</v>
       </c>
       <c r="C201">
         <v>1</v>
@@ -5741,10 +5747,10 @@
     </row>
     <row r="202" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A202" t="s">
-        <v>651</v>
+        <v>650</v>
       </c>
       <c r="B202" t="s">
-        <v>1010</v>
+        <v>1009</v>
       </c>
     </row>
     <row r="203" spans="1:3" x14ac:dyDescent="0.3">
@@ -5754,7 +5760,7 @@
     </row>
     <row r="204" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A204" t="s">
-        <v>652</v>
+        <v>651</v>
       </c>
     </row>
     <row r="205" spans="1:3" x14ac:dyDescent="0.3">
@@ -5769,12 +5775,12 @@
     </row>
     <row r="207" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A207" t="s">
-        <v>653</v>
+        <v>652</v>
       </c>
     </row>
     <row r="208" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A208" t="s">
-        <v>654</v>
+        <v>653</v>
       </c>
     </row>
     <row r="209" spans="1:6" x14ac:dyDescent="0.3">
@@ -5784,7 +5790,7 @@
       <c r="B209" s="8"/>
       <c r="C209" s="5">
         <f>SUM(C2:C208)</f>
-        <v>8</v>
+        <v>9</v>
       </c>
       <c r="D209" s="5">
         <f>SUM(D2:D208)</f>
@@ -5792,27 +5798,27 @@
       </c>
       <c r="E209" s="5">
         <f>SUM(E2:E208)</f>
-        <v>54</v>
+        <v>52</v>
       </c>
       <c r="F209" s="6" t="s">
-        <v>1012</v>
+        <v>1014</v>
       </c>
     </row>
     <row r="210" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A210" t="s">
-        <v>655</v>
+        <v>654</v>
       </c>
       <c r="B210" s="9"/>
       <c r="C210" s="4"/>
       <c r="D210" s="4"/>
       <c r="E210" s="4"/>
       <c r="F210" s="7" t="s">
-        <v>1014</v>
+        <v>1015</v>
       </c>
     </row>
     <row r="211" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A211" t="s">
-        <v>656</v>
+        <v>655</v>
       </c>
     </row>
     <row r="212" spans="1:6" x14ac:dyDescent="0.3">
@@ -5857,22 +5863,22 @@
     </row>
     <row r="220" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A220" t="s">
-        <v>657</v>
+        <v>656</v>
       </c>
     </row>
     <row r="221" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A221" t="s">
-        <v>658</v>
+        <v>657</v>
       </c>
     </row>
     <row r="222" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A222" t="s">
-        <v>659</v>
+        <v>658</v>
       </c>
     </row>
     <row r="223" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A223" t="s">
-        <v>660</v>
+        <v>659</v>
       </c>
     </row>
     <row r="224" spans="1:6" x14ac:dyDescent="0.3">
@@ -5882,12 +5888,12 @@
     </row>
     <row r="225" spans="1:1" x14ac:dyDescent="0.3">
       <c r="A225" t="s">
-        <v>661</v>
+        <v>660</v>
       </c>
     </row>
     <row r="226" spans="1:1" x14ac:dyDescent="0.3">
       <c r="A226" t="s">
-        <v>662</v>
+        <v>661</v>
       </c>
     </row>
     <row r="227" spans="1:1" x14ac:dyDescent="0.3">
@@ -5907,27 +5913,27 @@
     </row>
     <row r="230" spans="1:1" x14ac:dyDescent="0.3">
       <c r="A230" t="s">
-        <v>663</v>
+        <v>662</v>
       </c>
     </row>
     <row r="231" spans="1:1" x14ac:dyDescent="0.3">
       <c r="A231" t="s">
-        <v>664</v>
+        <v>663</v>
       </c>
     </row>
     <row r="232" spans="1:1" x14ac:dyDescent="0.3">
       <c r="A232" t="s">
-        <v>665</v>
+        <v>664</v>
       </c>
     </row>
     <row r="233" spans="1:1" x14ac:dyDescent="0.3">
       <c r="A233" t="s">
-        <v>666</v>
+        <v>665</v>
       </c>
     </row>
     <row r="234" spans="1:1" x14ac:dyDescent="0.3">
       <c r="A234" t="s">
-        <v>608</v>
+        <v>607</v>
       </c>
     </row>
     <row r="235" spans="1:1" x14ac:dyDescent="0.3">
@@ -5937,17 +5943,17 @@
     </row>
     <row r="236" spans="1:1" x14ac:dyDescent="0.3">
       <c r="A236" t="s">
-        <v>667</v>
+        <v>666</v>
       </c>
     </row>
     <row r="237" spans="1:1" x14ac:dyDescent="0.3">
       <c r="A237" t="s">
-        <v>668</v>
+        <v>667</v>
       </c>
     </row>
     <row r="238" spans="1:1" x14ac:dyDescent="0.3">
       <c r="A238" t="s">
-        <v>669</v>
+        <v>668</v>
       </c>
     </row>
     <row r="239" spans="1:1" x14ac:dyDescent="0.3">
@@ -5957,17 +5963,17 @@
     </row>
     <row r="240" spans="1:1" x14ac:dyDescent="0.3">
       <c r="A240" t="s">
-        <v>670</v>
+        <v>669</v>
       </c>
     </row>
     <row r="241" spans="1:1" x14ac:dyDescent="0.3">
       <c r="A241" t="s">
-        <v>671</v>
+        <v>670</v>
       </c>
     </row>
     <row r="242" spans="1:1" x14ac:dyDescent="0.3">
       <c r="A242" t="s">
-        <v>672</v>
+        <v>671</v>
       </c>
     </row>
     <row r="243" spans="1:1" x14ac:dyDescent="0.3">
@@ -5977,7 +5983,7 @@
     </row>
     <row r="244" spans="1:1" x14ac:dyDescent="0.3">
       <c r="A244" t="s">
-        <v>673</v>
+        <v>672</v>
       </c>
     </row>
     <row r="245" spans="1:1" x14ac:dyDescent="0.3">
@@ -5992,12 +5998,12 @@
     </row>
     <row r="247" spans="1:1" x14ac:dyDescent="0.3">
       <c r="A247" t="s">
-        <v>674</v>
+        <v>673</v>
       </c>
     </row>
     <row r="248" spans="1:1" x14ac:dyDescent="0.3">
       <c r="A248" t="s">
-        <v>675</v>
+        <v>674</v>
       </c>
     </row>
     <row r="249" spans="1:1" x14ac:dyDescent="0.3">
@@ -6007,17 +6013,17 @@
     </row>
     <row r="250" spans="1:1" x14ac:dyDescent="0.3">
       <c r="A250" t="s">
-        <v>676</v>
+        <v>675</v>
       </c>
     </row>
     <row r="251" spans="1:1" x14ac:dyDescent="0.3">
       <c r="A251" t="s">
-        <v>677</v>
+        <v>676</v>
       </c>
     </row>
     <row r="252" spans="1:1" x14ac:dyDescent="0.3">
       <c r="A252" t="s">
-        <v>678</v>
+        <v>677</v>
       </c>
     </row>
     <row r="253" spans="1:1" x14ac:dyDescent="0.3">
@@ -6027,7 +6033,7 @@
     </row>
     <row r="254" spans="1:1" x14ac:dyDescent="0.3">
       <c r="A254" t="s">
-        <v>679</v>
+        <v>678</v>
       </c>
     </row>
     <row r="255" spans="1:1" x14ac:dyDescent="0.3">
@@ -6047,12 +6053,12 @@
     </row>
     <row r="258" spans="1:1" x14ac:dyDescent="0.3">
       <c r="A258" t="s">
-        <v>680</v>
+        <v>679</v>
       </c>
     </row>
     <row r="259" spans="1:1" x14ac:dyDescent="0.3">
       <c r="A259" t="s">
-        <v>681</v>
+        <v>680</v>
       </c>
     </row>
     <row r="260" spans="1:1" x14ac:dyDescent="0.3">
@@ -6077,7 +6083,7 @@
     </row>
     <row r="264" spans="1:1" x14ac:dyDescent="0.3">
       <c r="A264" t="s">
-        <v>682</v>
+        <v>681</v>
       </c>
     </row>
     <row r="265" spans="1:1" x14ac:dyDescent="0.3">
@@ -6097,7 +6103,7 @@
     </row>
     <row r="268" spans="1:1" x14ac:dyDescent="0.3">
       <c r="A268" t="s">
-        <v>683</v>
+        <v>682</v>
       </c>
     </row>
     <row r="269" spans="1:1" x14ac:dyDescent="0.3">
@@ -6127,17 +6133,17 @@
     </row>
     <row r="274" spans="1:1" x14ac:dyDescent="0.3">
       <c r="A274" t="s">
-        <v>684</v>
+        <v>683</v>
       </c>
     </row>
     <row r="275" spans="1:1" x14ac:dyDescent="0.3">
       <c r="A275" t="s">
-        <v>685</v>
+        <v>684</v>
       </c>
     </row>
     <row r="276" spans="1:1" x14ac:dyDescent="0.3">
       <c r="A276" t="s">
-        <v>686</v>
+        <v>685</v>
       </c>
     </row>
     <row r="277" spans="1:1" x14ac:dyDescent="0.3">
@@ -6147,12 +6153,12 @@
     </row>
     <row r="278" spans="1:1" x14ac:dyDescent="0.3">
       <c r="A278" t="s">
-        <v>687</v>
+        <v>686</v>
       </c>
     </row>
     <row r="279" spans="1:1" x14ac:dyDescent="0.3">
       <c r="A279" t="s">
-        <v>688</v>
+        <v>687</v>
       </c>
     </row>
     <row r="280" spans="1:1" x14ac:dyDescent="0.3">
@@ -6162,37 +6168,37 @@
     </row>
     <row r="281" spans="1:1" x14ac:dyDescent="0.3">
       <c r="A281" t="s">
-        <v>689</v>
+        <v>688</v>
       </c>
     </row>
     <row r="282" spans="1:1" x14ac:dyDescent="0.3">
       <c r="A282" t="s">
-        <v>690</v>
+        <v>689</v>
       </c>
     </row>
     <row r="283" spans="1:1" x14ac:dyDescent="0.3">
       <c r="A283" t="s">
-        <v>691</v>
+        <v>690</v>
       </c>
     </row>
     <row r="284" spans="1:1" x14ac:dyDescent="0.3">
       <c r="A284" t="s">
-        <v>692</v>
+        <v>691</v>
       </c>
     </row>
     <row r="285" spans="1:1" x14ac:dyDescent="0.3">
       <c r="A285" t="s">
-        <v>693</v>
+        <v>692</v>
       </c>
     </row>
     <row r="286" spans="1:1" x14ac:dyDescent="0.3">
       <c r="A286" t="s">
-        <v>694</v>
+        <v>693</v>
       </c>
     </row>
     <row r="287" spans="1:1" x14ac:dyDescent="0.3">
       <c r="A287" t="s">
-        <v>695</v>
+        <v>694</v>
       </c>
     </row>
     <row r="288" spans="1:1" x14ac:dyDescent="0.3">
@@ -6207,12 +6213,12 @@
     </row>
     <row r="290" spans="1:1" x14ac:dyDescent="0.3">
       <c r="A290" t="s">
-        <v>669</v>
+        <v>668</v>
       </c>
     </row>
     <row r="291" spans="1:1" x14ac:dyDescent="0.3">
       <c r="A291" t="s">
-        <v>696</v>
+        <v>695</v>
       </c>
     </row>
     <row r="292" spans="1:1" x14ac:dyDescent="0.3">
@@ -6247,12 +6253,12 @@
     </row>
     <row r="298" spans="1:1" x14ac:dyDescent="0.3">
       <c r="A298" t="s">
-        <v>697</v>
+        <v>696</v>
       </c>
     </row>
     <row r="299" spans="1:1" x14ac:dyDescent="0.3">
       <c r="A299" t="s">
-        <v>698</v>
+        <v>697</v>
       </c>
     </row>
     <row r="300" spans="1:1" x14ac:dyDescent="0.3">
@@ -6262,12 +6268,12 @@
     </row>
     <row r="301" spans="1:1" x14ac:dyDescent="0.3">
       <c r="A301" t="s">
-        <v>669</v>
+        <v>668</v>
       </c>
     </row>
     <row r="302" spans="1:1" x14ac:dyDescent="0.3">
       <c r="A302" t="s">
-        <v>699</v>
+        <v>698</v>
       </c>
     </row>
     <row r="303" spans="1:1" x14ac:dyDescent="0.3">
@@ -6282,7 +6288,7 @@
     </row>
     <row r="305" spans="1:1" x14ac:dyDescent="0.3">
       <c r="A305" t="s">
-        <v>700</v>
+        <v>699</v>
       </c>
     </row>
     <row r="306" spans="1:1" x14ac:dyDescent="0.3">
@@ -6312,17 +6318,17 @@
     </row>
     <row r="311" spans="1:1" x14ac:dyDescent="0.3">
       <c r="A311" t="s">
-        <v>701</v>
+        <v>700</v>
       </c>
     </row>
     <row r="312" spans="1:1" x14ac:dyDescent="0.3">
       <c r="A312" t="s">
-        <v>702</v>
+        <v>701</v>
       </c>
     </row>
     <row r="313" spans="1:1" x14ac:dyDescent="0.3">
       <c r="A313" t="s">
-        <v>703</v>
+        <v>702</v>
       </c>
     </row>
     <row r="314" spans="1:1" x14ac:dyDescent="0.3">
@@ -6332,7 +6338,7 @@
     </row>
     <row r="315" spans="1:1" x14ac:dyDescent="0.3">
       <c r="A315" t="s">
-        <v>704</v>
+        <v>703</v>
       </c>
     </row>
     <row r="316" spans="1:1" x14ac:dyDescent="0.3">
@@ -6342,7 +6348,7 @@
     </row>
     <row r="317" spans="1:1" x14ac:dyDescent="0.3">
       <c r="A317" t="s">
-        <v>705</v>
+        <v>704</v>
       </c>
     </row>
     <row r="318" spans="1:1" x14ac:dyDescent="0.3">
@@ -6352,7 +6358,7 @@
     </row>
     <row r="319" spans="1:1" x14ac:dyDescent="0.3">
       <c r="A319" t="s">
-        <v>706</v>
+        <v>705</v>
       </c>
     </row>
     <row r="320" spans="1:1" x14ac:dyDescent="0.3">
@@ -6372,12 +6378,12 @@
     </row>
     <row r="323" spans="1:1" x14ac:dyDescent="0.3">
       <c r="A323" t="s">
-        <v>707</v>
+        <v>706</v>
       </c>
     </row>
     <row r="324" spans="1:1" x14ac:dyDescent="0.3">
       <c r="A324" t="s">
-        <v>708</v>
+        <v>707</v>
       </c>
     </row>
     <row r="325" spans="1:1" x14ac:dyDescent="0.3">
@@ -6387,7 +6393,7 @@
     </row>
     <row r="326" spans="1:1" x14ac:dyDescent="0.3">
       <c r="A326" t="s">
-        <v>709</v>
+        <v>708</v>
       </c>
     </row>
     <row r="327" spans="1:1" x14ac:dyDescent="0.3">
@@ -6402,7 +6408,7 @@
     </row>
     <row r="329" spans="1:1" x14ac:dyDescent="0.3">
       <c r="A329" t="s">
-        <v>710</v>
+        <v>709</v>
       </c>
     </row>
     <row r="330" spans="1:1" x14ac:dyDescent="0.3">
@@ -6412,17 +6418,17 @@
     </row>
     <row r="331" spans="1:1" x14ac:dyDescent="0.3">
       <c r="A331" t="s">
-        <v>711</v>
+        <v>710</v>
       </c>
     </row>
     <row r="332" spans="1:1" x14ac:dyDescent="0.3">
       <c r="A332" t="s">
-        <v>711</v>
+        <v>710</v>
       </c>
     </row>
     <row r="333" spans="1:1" x14ac:dyDescent="0.3">
       <c r="A333" t="s">
-        <v>712</v>
+        <v>711</v>
       </c>
     </row>
     <row r="334" spans="1:1" x14ac:dyDescent="0.3">
@@ -6442,32 +6448,32 @@
     </row>
     <row r="337" spans="1:1" x14ac:dyDescent="0.3">
       <c r="A337" t="s">
-        <v>713</v>
+        <v>712</v>
       </c>
     </row>
     <row r="338" spans="1:1" x14ac:dyDescent="0.3">
       <c r="A338" t="s">
-        <v>714</v>
+        <v>713</v>
       </c>
     </row>
     <row r="339" spans="1:1" x14ac:dyDescent="0.3">
       <c r="A339" t="s">
-        <v>715</v>
+        <v>714</v>
       </c>
     </row>
     <row r="340" spans="1:1" x14ac:dyDescent="0.3">
       <c r="A340" t="s">
-        <v>716</v>
+        <v>715</v>
       </c>
     </row>
     <row r="341" spans="1:1" x14ac:dyDescent="0.3">
       <c r="A341" t="s">
-        <v>717</v>
+        <v>716</v>
       </c>
     </row>
     <row r="342" spans="1:1" x14ac:dyDescent="0.3">
       <c r="A342" t="s">
-        <v>718</v>
+        <v>717</v>
       </c>
     </row>
     <row r="343" spans="1:1" x14ac:dyDescent="0.3">
@@ -6477,7 +6483,7 @@
     </row>
     <row r="344" spans="1:1" x14ac:dyDescent="0.3">
       <c r="A344" t="s">
-        <v>719</v>
+        <v>718</v>
       </c>
     </row>
     <row r="345" spans="1:1" x14ac:dyDescent="0.3">
@@ -6497,7 +6503,7 @@
     </row>
     <row r="348" spans="1:1" x14ac:dyDescent="0.3">
       <c r="A348" t="s">
-        <v>720</v>
+        <v>719</v>
       </c>
     </row>
     <row r="349" spans="1:1" x14ac:dyDescent="0.3">
@@ -6522,7 +6528,7 @@
     </row>
     <row r="353" spans="1:1" x14ac:dyDescent="0.3">
       <c r="A353" t="s">
-        <v>721</v>
+        <v>720</v>
       </c>
     </row>
     <row r="354" spans="1:1" x14ac:dyDescent="0.3">
@@ -6532,7 +6538,7 @@
     </row>
     <row r="355" spans="1:1" x14ac:dyDescent="0.3">
       <c r="A355" t="s">
-        <v>722</v>
+        <v>721</v>
       </c>
     </row>
     <row r="356" spans="1:1" x14ac:dyDescent="0.3">
@@ -6547,7 +6553,7 @@
     </row>
     <row r="358" spans="1:1" x14ac:dyDescent="0.3">
       <c r="A358" t="s">
-        <v>723</v>
+        <v>722</v>
       </c>
     </row>
     <row r="359" spans="1:1" x14ac:dyDescent="0.3">
@@ -6557,17 +6563,17 @@
     </row>
     <row r="360" spans="1:1" x14ac:dyDescent="0.3">
       <c r="A360" t="s">
-        <v>724</v>
+        <v>723</v>
       </c>
     </row>
     <row r="361" spans="1:1" x14ac:dyDescent="0.3">
       <c r="A361" t="s">
-        <v>725</v>
+        <v>724</v>
       </c>
     </row>
     <row r="362" spans="1:1" x14ac:dyDescent="0.3">
       <c r="A362" t="s">
-        <v>726</v>
+        <v>725</v>
       </c>
     </row>
     <row r="363" spans="1:1" x14ac:dyDescent="0.3">
@@ -6622,7 +6628,7 @@
     </row>
     <row r="373" spans="1:1" x14ac:dyDescent="0.3">
       <c r="A373" t="s">
-        <v>727</v>
+        <v>726</v>
       </c>
     </row>
     <row r="374" spans="1:1" x14ac:dyDescent="0.3">
@@ -6637,12 +6643,12 @@
     </row>
     <row r="376" spans="1:1" x14ac:dyDescent="0.3">
       <c r="A376" t="s">
-        <v>728</v>
+        <v>727</v>
       </c>
     </row>
     <row r="377" spans="1:1" x14ac:dyDescent="0.3">
       <c r="A377" t="s">
-        <v>729</v>
+        <v>728</v>
       </c>
     </row>
     <row r="378" spans="1:1" x14ac:dyDescent="0.3">
@@ -6667,22 +6673,22 @@
     </row>
     <row r="382" spans="1:1" x14ac:dyDescent="0.3">
       <c r="A382" t="s">
-        <v>730</v>
+        <v>729</v>
       </c>
     </row>
     <row r="383" spans="1:1" x14ac:dyDescent="0.3">
       <c r="A383" t="s">
-        <v>731</v>
+        <v>730</v>
       </c>
     </row>
     <row r="384" spans="1:1" x14ac:dyDescent="0.3">
       <c r="A384" t="s">
-        <v>732</v>
+        <v>731</v>
       </c>
     </row>
     <row r="385" spans="1:1" x14ac:dyDescent="0.3">
       <c r="A385" t="s">
-        <v>733</v>
+        <v>732</v>
       </c>
     </row>
     <row r="386" spans="1:1" x14ac:dyDescent="0.3">
@@ -6707,17 +6713,17 @@
     </row>
     <row r="390" spans="1:1" x14ac:dyDescent="0.3">
       <c r="A390" t="s">
-        <v>734</v>
+        <v>733</v>
       </c>
     </row>
     <row r="391" spans="1:1" x14ac:dyDescent="0.3">
       <c r="A391" t="s">
-        <v>735</v>
+        <v>734</v>
       </c>
     </row>
     <row r="392" spans="1:1" x14ac:dyDescent="0.3">
       <c r="A392" t="s">
-        <v>736</v>
+        <v>735</v>
       </c>
     </row>
     <row r="393" spans="1:1" x14ac:dyDescent="0.3">
@@ -6727,7 +6733,7 @@
     </row>
     <row r="394" spans="1:1" x14ac:dyDescent="0.3">
       <c r="A394" t="s">
-        <v>737</v>
+        <v>736</v>
       </c>
     </row>
     <row r="395" spans="1:1" x14ac:dyDescent="0.3">
@@ -6767,7 +6773,7 @@
     </row>
     <row r="402" spans="1:1" x14ac:dyDescent="0.3">
       <c r="A402" t="s">
-        <v>738</v>
+        <v>737</v>
       </c>
     </row>
     <row r="403" spans="1:1" x14ac:dyDescent="0.3">
@@ -6777,12 +6783,12 @@
     </row>
     <row r="404" spans="1:1" x14ac:dyDescent="0.3">
       <c r="A404" t="s">
-        <v>739</v>
+        <v>738</v>
       </c>
     </row>
     <row r="405" spans="1:1" x14ac:dyDescent="0.3">
       <c r="A405" t="s">
-        <v>740</v>
+        <v>739</v>
       </c>
     </row>
     <row r="406" spans="1:1" x14ac:dyDescent="0.3">
@@ -6792,7 +6798,7 @@
     </row>
     <row r="407" spans="1:1" x14ac:dyDescent="0.3">
       <c r="A407" t="s">
-        <v>741</v>
+        <v>740</v>
       </c>
     </row>
     <row r="408" spans="1:1" x14ac:dyDescent="0.3">
@@ -6802,12 +6808,12 @@
     </row>
     <row r="409" spans="1:1" x14ac:dyDescent="0.3">
       <c r="A409" t="s">
-        <v>742</v>
+        <v>741</v>
       </c>
     </row>
     <row r="410" spans="1:1" x14ac:dyDescent="0.3">
       <c r="A410" t="s">
-        <v>743</v>
+        <v>742</v>
       </c>
     </row>
     <row r="411" spans="1:1" x14ac:dyDescent="0.3">
@@ -6852,7 +6858,7 @@
     </row>
     <row r="419" spans="1:1" x14ac:dyDescent="0.3">
       <c r="A419" t="s">
-        <v>744</v>
+        <v>743</v>
       </c>
     </row>
     <row r="420" spans="1:1" x14ac:dyDescent="0.3">
@@ -6862,22 +6868,22 @@
     </row>
     <row r="421" spans="1:1" x14ac:dyDescent="0.3">
       <c r="A421" t="s">
-        <v>745</v>
+        <v>744</v>
       </c>
     </row>
     <row r="422" spans="1:1" x14ac:dyDescent="0.3">
       <c r="A422" t="s">
-        <v>746</v>
+        <v>745</v>
       </c>
     </row>
     <row r="423" spans="1:1" x14ac:dyDescent="0.3">
       <c r="A423" t="s">
-        <v>746</v>
+        <v>745</v>
       </c>
     </row>
     <row r="424" spans="1:1" x14ac:dyDescent="0.3">
       <c r="A424" t="s">
-        <v>747</v>
+        <v>746</v>
       </c>
     </row>
     <row r="425" spans="1:1" x14ac:dyDescent="0.3">
@@ -6897,17 +6903,17 @@
     </row>
     <row r="428" spans="1:1" x14ac:dyDescent="0.3">
       <c r="A428" t="s">
-        <v>748</v>
+        <v>747</v>
       </c>
     </row>
     <row r="429" spans="1:1" x14ac:dyDescent="0.3">
       <c r="A429" t="s">
-        <v>749</v>
+        <v>748</v>
       </c>
     </row>
     <row r="430" spans="1:1" x14ac:dyDescent="0.3">
       <c r="A430" t="s">
-        <v>750</v>
+        <v>749</v>
       </c>
     </row>
     <row r="431" spans="1:1" x14ac:dyDescent="0.3">
@@ -6917,7 +6923,7 @@
     </row>
     <row r="432" spans="1:1" x14ac:dyDescent="0.3">
       <c r="A432" t="s">
-        <v>751</v>
+        <v>750</v>
       </c>
     </row>
     <row r="433" spans="1:1" x14ac:dyDescent="0.3">
@@ -6937,12 +6943,12 @@
     </row>
     <row r="436" spans="1:1" x14ac:dyDescent="0.3">
       <c r="A436" t="s">
-        <v>752</v>
+        <v>751</v>
       </c>
     </row>
     <row r="437" spans="1:1" x14ac:dyDescent="0.3">
       <c r="A437" t="s">
-        <v>753</v>
+        <v>752</v>
       </c>
     </row>
     <row r="438" spans="1:1" x14ac:dyDescent="0.3">
@@ -6952,7 +6958,7 @@
     </row>
     <row r="439" spans="1:1" x14ac:dyDescent="0.3">
       <c r="A439" t="s">
-        <v>754</v>
+        <v>753</v>
       </c>
     </row>
     <row r="440" spans="1:1" x14ac:dyDescent="0.3">
@@ -6967,17 +6973,17 @@
     </row>
     <row r="442" spans="1:1" x14ac:dyDescent="0.3">
       <c r="A442" t="s">
-        <v>702</v>
+        <v>701</v>
       </c>
     </row>
     <row r="443" spans="1:1" x14ac:dyDescent="0.3">
       <c r="A443" t="s">
-        <v>755</v>
+        <v>754</v>
       </c>
     </row>
     <row r="444" spans="1:1" x14ac:dyDescent="0.3">
       <c r="A444" t="s">
-        <v>756</v>
+        <v>755</v>
       </c>
     </row>
     <row r="445" spans="1:1" x14ac:dyDescent="0.3">
@@ -6997,17 +7003,17 @@
     </row>
     <row r="448" spans="1:1" x14ac:dyDescent="0.3">
       <c r="A448" t="s">
-        <v>757</v>
+        <v>756</v>
       </c>
     </row>
     <row r="449" spans="1:1" x14ac:dyDescent="0.3">
       <c r="A449" t="s">
-        <v>758</v>
+        <v>757</v>
       </c>
     </row>
     <row r="450" spans="1:1" x14ac:dyDescent="0.3">
       <c r="A450" t="s">
-        <v>759</v>
+        <v>758</v>
       </c>
     </row>
     <row r="451" spans="1:1" x14ac:dyDescent="0.3">
@@ -7017,7 +7023,7 @@
     </row>
     <row r="452" spans="1:1" x14ac:dyDescent="0.3">
       <c r="A452" t="s">
-        <v>760</v>
+        <v>759</v>
       </c>
     </row>
     <row r="453" spans="1:1" x14ac:dyDescent="0.3">
@@ -7032,7 +7038,7 @@
     </row>
     <row r="455" spans="1:1" x14ac:dyDescent="0.3">
       <c r="A455" t="s">
-        <v>761</v>
+        <v>760</v>
       </c>
     </row>
     <row r="456" spans="1:1" x14ac:dyDescent="0.3">
@@ -7042,7 +7048,7 @@
     </row>
     <row r="457" spans="1:1" x14ac:dyDescent="0.3">
       <c r="A457" t="s">
-        <v>762</v>
+        <v>761</v>
       </c>
     </row>
     <row r="458" spans="1:1" x14ac:dyDescent="0.3">
@@ -7057,7 +7063,7 @@
     </row>
     <row r="460" spans="1:1" x14ac:dyDescent="0.3">
       <c r="A460" t="s">
-        <v>763</v>
+        <v>762</v>
       </c>
     </row>
     <row r="461" spans="1:1" x14ac:dyDescent="0.3">
@@ -7072,7 +7078,7 @@
     </row>
     <row r="463" spans="1:1" x14ac:dyDescent="0.3">
       <c r="A463" t="s">
-        <v>764</v>
+        <v>763</v>
       </c>
     </row>
     <row r="464" spans="1:1" x14ac:dyDescent="0.3">
@@ -7082,17 +7088,17 @@
     </row>
     <row r="465" spans="1:1" x14ac:dyDescent="0.3">
       <c r="A465" t="s">
-        <v>765</v>
+        <v>764</v>
       </c>
     </row>
     <row r="466" spans="1:1" x14ac:dyDescent="0.3">
       <c r="A466" t="s">
-        <v>766</v>
+        <v>765</v>
       </c>
     </row>
     <row r="467" spans="1:1" x14ac:dyDescent="0.3">
       <c r="A467" t="s">
-        <v>767</v>
+        <v>766</v>
       </c>
     </row>
     <row r="468" spans="1:1" x14ac:dyDescent="0.3">
@@ -7102,7 +7108,7 @@
     </row>
     <row r="469" spans="1:1" x14ac:dyDescent="0.3">
       <c r="A469" t="s">
-        <v>768</v>
+        <v>767</v>
       </c>
     </row>
     <row r="470" spans="1:1" x14ac:dyDescent="0.3">
@@ -7112,17 +7118,17 @@
     </row>
     <row r="471" spans="1:1" x14ac:dyDescent="0.3">
       <c r="A471" t="s">
-        <v>769</v>
+        <v>768</v>
       </c>
     </row>
     <row r="472" spans="1:1" x14ac:dyDescent="0.3">
       <c r="A472" t="s">
-        <v>770</v>
+        <v>769</v>
       </c>
     </row>
     <row r="473" spans="1:1" x14ac:dyDescent="0.3">
       <c r="A473" t="s">
-        <v>771</v>
+        <v>770</v>
       </c>
     </row>
     <row r="474" spans="1:1" x14ac:dyDescent="0.3">
@@ -7137,7 +7143,7 @@
     </row>
     <row r="476" spans="1:1" x14ac:dyDescent="0.3">
       <c r="A476" t="s">
-        <v>772</v>
+        <v>771</v>
       </c>
     </row>
     <row r="477" spans="1:1" x14ac:dyDescent="0.3">
@@ -7147,7 +7153,7 @@
     </row>
     <row r="478" spans="1:1" x14ac:dyDescent="0.3">
       <c r="A478" t="s">
-        <v>773</v>
+        <v>772</v>
       </c>
     </row>
     <row r="479" spans="1:1" x14ac:dyDescent="0.3">
@@ -7157,22 +7163,22 @@
     </row>
     <row r="480" spans="1:1" x14ac:dyDescent="0.3">
       <c r="A480" t="s">
-        <v>774</v>
+        <v>773</v>
       </c>
     </row>
     <row r="481" spans="1:1" x14ac:dyDescent="0.3">
       <c r="A481" t="s">
-        <v>775</v>
+        <v>774</v>
       </c>
     </row>
     <row r="482" spans="1:1" x14ac:dyDescent="0.3">
       <c r="A482" t="s">
-        <v>776</v>
+        <v>775</v>
       </c>
     </row>
     <row r="483" spans="1:1" x14ac:dyDescent="0.3">
       <c r="A483" t="s">
-        <v>777</v>
+        <v>776</v>
       </c>
     </row>
     <row r="484" spans="1:1" x14ac:dyDescent="0.3">
@@ -7192,7 +7198,7 @@
     </row>
     <row r="487" spans="1:1" x14ac:dyDescent="0.3">
       <c r="A487" t="s">
-        <v>778</v>
+        <v>777</v>
       </c>
     </row>
     <row r="488" spans="1:1" x14ac:dyDescent="0.3">
@@ -7207,37 +7213,37 @@
     </row>
     <row r="490" spans="1:1" x14ac:dyDescent="0.3">
       <c r="A490" t="s">
-        <v>779</v>
+        <v>778</v>
       </c>
     </row>
     <row r="491" spans="1:1" x14ac:dyDescent="0.3">
       <c r="A491" t="s">
-        <v>780</v>
+        <v>779</v>
       </c>
     </row>
     <row r="492" spans="1:1" x14ac:dyDescent="0.3">
       <c r="A492" t="s">
-        <v>781</v>
+        <v>780</v>
       </c>
     </row>
     <row r="493" spans="1:1" x14ac:dyDescent="0.3">
       <c r="A493" t="s">
-        <v>782</v>
+        <v>781</v>
       </c>
     </row>
     <row r="494" spans="1:1" x14ac:dyDescent="0.3">
       <c r="A494" t="s">
-        <v>783</v>
+        <v>782</v>
       </c>
     </row>
     <row r="495" spans="1:1" x14ac:dyDescent="0.3">
       <c r="A495" t="s">
-        <v>784</v>
+        <v>783</v>
       </c>
     </row>
     <row r="496" spans="1:1" x14ac:dyDescent="0.3">
       <c r="A496" t="s">
-        <v>785</v>
+        <v>784</v>
       </c>
     </row>
     <row r="497" spans="1:1" x14ac:dyDescent="0.3">
@@ -7247,27 +7253,27 @@
     </row>
     <row r="498" spans="1:1" x14ac:dyDescent="0.3">
       <c r="A498" t="s">
-        <v>786</v>
+        <v>785</v>
       </c>
     </row>
     <row r="499" spans="1:1" x14ac:dyDescent="0.3">
       <c r="A499" t="s">
-        <v>787</v>
+        <v>786</v>
       </c>
     </row>
     <row r="500" spans="1:1" x14ac:dyDescent="0.3">
       <c r="A500" t="s">
-        <v>788</v>
+        <v>787</v>
       </c>
     </row>
     <row r="501" spans="1:1" x14ac:dyDescent="0.3">
       <c r="A501" t="s">
-        <v>789</v>
+        <v>788</v>
       </c>
     </row>
     <row r="502" spans="1:1" x14ac:dyDescent="0.3">
       <c r="A502" t="s">
-        <v>790</v>
+        <v>789</v>
       </c>
     </row>
     <row r="503" spans="1:1" x14ac:dyDescent="0.3">
@@ -7277,17 +7283,17 @@
     </row>
     <row r="504" spans="1:1" x14ac:dyDescent="0.3">
       <c r="A504" t="s">
-        <v>791</v>
+        <v>790</v>
       </c>
     </row>
     <row r="505" spans="1:1" x14ac:dyDescent="0.3">
       <c r="A505" t="s">
-        <v>792</v>
+        <v>791</v>
       </c>
     </row>
     <row r="506" spans="1:1" x14ac:dyDescent="0.3">
       <c r="A506" t="s">
-        <v>793</v>
+        <v>792</v>
       </c>
     </row>
     <row r="507" spans="1:1" x14ac:dyDescent="0.3">
@@ -7307,22 +7313,22 @@
     </row>
     <row r="510" spans="1:1" x14ac:dyDescent="0.3">
       <c r="A510" t="s">
-        <v>794</v>
+        <v>793</v>
       </c>
     </row>
     <row r="511" spans="1:1" x14ac:dyDescent="0.3">
       <c r="A511" t="s">
-        <v>795</v>
+        <v>794</v>
       </c>
     </row>
     <row r="512" spans="1:1" x14ac:dyDescent="0.3">
       <c r="A512" t="s">
-        <v>796</v>
+        <v>795</v>
       </c>
     </row>
     <row r="513" spans="1:1" x14ac:dyDescent="0.3">
       <c r="A513" t="s">
-        <v>797</v>
+        <v>796</v>
       </c>
     </row>
     <row r="514" spans="1:1" x14ac:dyDescent="0.3">
@@ -7332,27 +7338,27 @@
     </row>
     <row r="515" spans="1:1" x14ac:dyDescent="0.3">
       <c r="A515" t="s">
-        <v>798</v>
+        <v>797</v>
       </c>
     </row>
     <row r="516" spans="1:1" x14ac:dyDescent="0.3">
       <c r="A516" t="s">
-        <v>606</v>
+        <v>605</v>
       </c>
     </row>
     <row r="517" spans="1:1" x14ac:dyDescent="0.3">
       <c r="A517" t="s">
-        <v>799</v>
+        <v>798</v>
       </c>
     </row>
     <row r="518" spans="1:1" x14ac:dyDescent="0.3">
       <c r="A518" t="s">
-        <v>800</v>
+        <v>799</v>
       </c>
     </row>
     <row r="519" spans="1:1" x14ac:dyDescent="0.3">
       <c r="A519" t="s">
-        <v>801</v>
+        <v>800</v>
       </c>
     </row>
     <row r="520" spans="1:1" x14ac:dyDescent="0.3">
@@ -7362,7 +7368,7 @@
     </row>
     <row r="521" spans="1:1" x14ac:dyDescent="0.3">
       <c r="A521" t="s">
-        <v>802</v>
+        <v>801</v>
       </c>
     </row>
     <row r="522" spans="1:1" x14ac:dyDescent="0.3">
@@ -7372,12 +7378,12 @@
     </row>
     <row r="523" spans="1:1" x14ac:dyDescent="0.3">
       <c r="A523" t="s">
-        <v>803</v>
+        <v>802</v>
       </c>
     </row>
     <row r="524" spans="1:1" x14ac:dyDescent="0.3">
       <c r="A524" t="s">
-        <v>804</v>
+        <v>803</v>
       </c>
     </row>
     <row r="525" spans="1:1" x14ac:dyDescent="0.3">
@@ -7397,12 +7403,12 @@
     </row>
     <row r="528" spans="1:1" x14ac:dyDescent="0.3">
       <c r="A528" t="s">
-        <v>805</v>
+        <v>804</v>
       </c>
     </row>
     <row r="529" spans="1:1" x14ac:dyDescent="0.3">
       <c r="A529" t="s">
-        <v>806</v>
+        <v>805</v>
       </c>
     </row>
     <row r="530" spans="1:1" x14ac:dyDescent="0.3">
@@ -7437,7 +7443,7 @@
     </row>
     <row r="536" spans="1:1" x14ac:dyDescent="0.3">
       <c r="A536" t="s">
-        <v>807</v>
+        <v>806</v>
       </c>
     </row>
     <row r="537" spans="1:1" x14ac:dyDescent="0.3">
@@ -7447,7 +7453,7 @@
     </row>
     <row r="538" spans="1:1" x14ac:dyDescent="0.3">
       <c r="A538" t="s">
-        <v>808</v>
+        <v>807</v>
       </c>
     </row>
     <row r="539" spans="1:1" x14ac:dyDescent="0.3">
@@ -7457,27 +7463,27 @@
     </row>
     <row r="540" spans="1:1" x14ac:dyDescent="0.3">
       <c r="A540" t="s">
-        <v>809</v>
+        <v>808</v>
       </c>
     </row>
     <row r="541" spans="1:1" x14ac:dyDescent="0.3">
       <c r="A541" t="s">
-        <v>810</v>
+        <v>809</v>
       </c>
     </row>
     <row r="542" spans="1:1" x14ac:dyDescent="0.3">
       <c r="A542" t="s">
-        <v>811</v>
+        <v>810</v>
       </c>
     </row>
     <row r="543" spans="1:1" x14ac:dyDescent="0.3">
       <c r="A543" t="s">
-        <v>811</v>
+        <v>810</v>
       </c>
     </row>
     <row r="544" spans="1:1" x14ac:dyDescent="0.3">
       <c r="A544" t="s">
-        <v>812</v>
+        <v>811</v>
       </c>
     </row>
     <row r="545" spans="1:1" x14ac:dyDescent="0.3">
@@ -7487,12 +7493,12 @@
     </row>
     <row r="546" spans="1:1" x14ac:dyDescent="0.3">
       <c r="A546" t="s">
-        <v>813</v>
+        <v>812</v>
       </c>
     </row>
     <row r="547" spans="1:1" x14ac:dyDescent="0.3">
       <c r="A547" t="s">
-        <v>814</v>
+        <v>813</v>
       </c>
     </row>
     <row r="548" spans="1:1" x14ac:dyDescent="0.3">
@@ -7517,7 +7523,7 @@
     </row>
     <row r="552" spans="1:1" x14ac:dyDescent="0.3">
       <c r="A552" t="s">
-        <v>815</v>
+        <v>814</v>
       </c>
     </row>
     <row r="553" spans="1:1" x14ac:dyDescent="0.3">
@@ -7527,7 +7533,7 @@
     </row>
     <row r="554" spans="1:1" x14ac:dyDescent="0.3">
       <c r="A554" t="s">
-        <v>816</v>
+        <v>815</v>
       </c>
     </row>
     <row r="555" spans="1:1" x14ac:dyDescent="0.3">
@@ -7537,12 +7543,12 @@
     </row>
     <row r="556" spans="1:1" x14ac:dyDescent="0.3">
       <c r="A556" t="s">
-        <v>817</v>
+        <v>816</v>
       </c>
     </row>
     <row r="557" spans="1:1" x14ac:dyDescent="0.3">
       <c r="A557" t="s">
-        <v>818</v>
+        <v>817</v>
       </c>
     </row>
     <row r="558" spans="1:1" x14ac:dyDescent="0.3">
@@ -7552,7 +7558,7 @@
     </row>
     <row r="559" spans="1:1" x14ac:dyDescent="0.3">
       <c r="A559" t="s">
-        <v>819</v>
+        <v>818</v>
       </c>
     </row>
     <row r="560" spans="1:1" x14ac:dyDescent="0.3">
@@ -7562,7 +7568,7 @@
     </row>
     <row r="561" spans="1:1" x14ac:dyDescent="0.3">
       <c r="A561" t="s">
-        <v>820</v>
+        <v>819</v>
       </c>
     </row>
     <row r="562" spans="1:1" x14ac:dyDescent="0.3">
@@ -7577,17 +7583,17 @@
     </row>
     <row r="564" spans="1:1" x14ac:dyDescent="0.3">
       <c r="A564" t="s">
-        <v>821</v>
+        <v>820</v>
       </c>
     </row>
     <row r="565" spans="1:1" x14ac:dyDescent="0.3">
       <c r="A565" t="s">
-        <v>822</v>
+        <v>821</v>
       </c>
     </row>
     <row r="566" spans="1:1" x14ac:dyDescent="0.3">
       <c r="A566" t="s">
-        <v>823</v>
+        <v>822</v>
       </c>
     </row>
     <row r="567" spans="1:1" x14ac:dyDescent="0.3">
@@ -7602,7 +7608,7 @@
     </row>
     <row r="569" spans="1:1" x14ac:dyDescent="0.3">
       <c r="A569" t="s">
-        <v>824</v>
+        <v>823</v>
       </c>
     </row>
     <row r="570" spans="1:1" x14ac:dyDescent="0.3">
@@ -7612,27 +7618,27 @@
     </row>
     <row r="571" spans="1:1" x14ac:dyDescent="0.3">
       <c r="A571" t="s">
-        <v>825</v>
+        <v>824</v>
       </c>
     </row>
     <row r="572" spans="1:1" x14ac:dyDescent="0.3">
       <c r="A572" t="s">
-        <v>826</v>
+        <v>825</v>
       </c>
     </row>
     <row r="573" spans="1:1" x14ac:dyDescent="0.3">
       <c r="A573" t="s">
-        <v>827</v>
+        <v>826</v>
       </c>
     </row>
     <row r="574" spans="1:1" x14ac:dyDescent="0.3">
       <c r="A574" t="s">
-        <v>828</v>
+        <v>827</v>
       </c>
     </row>
     <row r="575" spans="1:1" x14ac:dyDescent="0.3">
       <c r="A575" t="s">
-        <v>829</v>
+        <v>828</v>
       </c>
     </row>
     <row r="576" spans="1:1" x14ac:dyDescent="0.3">
@@ -7657,7 +7663,7 @@
     </row>
     <row r="580" spans="1:1" x14ac:dyDescent="0.3">
       <c r="A580" t="s">
-        <v>830</v>
+        <v>829</v>
       </c>
     </row>
     <row r="581" spans="1:1" x14ac:dyDescent="0.3">
@@ -7692,7 +7698,7 @@
     </row>
     <row r="587" spans="1:1" x14ac:dyDescent="0.3">
       <c r="A587" t="s">
-        <v>831</v>
+        <v>830</v>
       </c>
     </row>
     <row r="588" spans="1:1" x14ac:dyDescent="0.3">
@@ -7712,7 +7718,7 @@
     </row>
     <row r="591" spans="1:1" x14ac:dyDescent="0.3">
       <c r="A591" t="s">
-        <v>832</v>
+        <v>831</v>
       </c>
     </row>
     <row r="592" spans="1:1" x14ac:dyDescent="0.3">
@@ -7727,7 +7733,7 @@
     </row>
     <row r="594" spans="1:1" x14ac:dyDescent="0.3">
       <c r="A594" t="s">
-        <v>833</v>
+        <v>832</v>
       </c>
     </row>
     <row r="595" spans="1:1" x14ac:dyDescent="0.3">
@@ -7747,7 +7753,7 @@
     </row>
     <row r="598" spans="1:1" x14ac:dyDescent="0.3">
       <c r="A598" t="s">
-        <v>834</v>
+        <v>833</v>
       </c>
     </row>
     <row r="599" spans="1:1" x14ac:dyDescent="0.3">
@@ -7762,17 +7768,17 @@
     </row>
     <row r="601" spans="1:1" x14ac:dyDescent="0.3">
       <c r="A601" t="s">
-        <v>835</v>
+        <v>834</v>
       </c>
     </row>
     <row r="602" spans="1:1" x14ac:dyDescent="0.3">
       <c r="A602" t="s">
-        <v>836</v>
+        <v>835</v>
       </c>
     </row>
     <row r="603" spans="1:1" x14ac:dyDescent="0.3">
       <c r="A603" t="s">
-        <v>837</v>
+        <v>836</v>
       </c>
     </row>
     <row r="604" spans="1:1" x14ac:dyDescent="0.3">
@@ -7782,12 +7788,12 @@
     </row>
     <row r="605" spans="1:1" x14ac:dyDescent="0.3">
       <c r="A605" t="s">
-        <v>838</v>
+        <v>837</v>
       </c>
     </row>
     <row r="606" spans="1:1" x14ac:dyDescent="0.3">
       <c r="A606" t="s">
-        <v>839</v>
+        <v>838</v>
       </c>
     </row>
     <row r="607" spans="1:1" x14ac:dyDescent="0.3">
@@ -7797,7 +7803,7 @@
     </row>
     <row r="608" spans="1:1" x14ac:dyDescent="0.3">
       <c r="A608" t="s">
-        <v>840</v>
+        <v>839</v>
       </c>
     </row>
     <row r="609" spans="1:1" x14ac:dyDescent="0.3">
@@ -7812,12 +7818,12 @@
     </row>
     <row r="611" spans="1:1" x14ac:dyDescent="0.3">
       <c r="A611" t="s">
-        <v>608</v>
+        <v>607</v>
       </c>
     </row>
     <row r="612" spans="1:1" x14ac:dyDescent="0.3">
       <c r="A612" t="s">
-        <v>841</v>
+        <v>840</v>
       </c>
     </row>
     <row r="613" spans="1:1" x14ac:dyDescent="0.3">
@@ -7832,17 +7838,17 @@
     </row>
     <row r="615" spans="1:1" x14ac:dyDescent="0.3">
       <c r="A615" t="s">
-        <v>842</v>
+        <v>841</v>
       </c>
     </row>
     <row r="616" spans="1:1" x14ac:dyDescent="0.3">
       <c r="A616" t="s">
-        <v>843</v>
+        <v>842</v>
       </c>
     </row>
     <row r="617" spans="1:1" x14ac:dyDescent="0.3">
       <c r="A617" t="s">
-        <v>844</v>
+        <v>843</v>
       </c>
     </row>
     <row r="618" spans="1:1" x14ac:dyDescent="0.3">
@@ -7852,12 +7858,12 @@
     </row>
     <row r="619" spans="1:1" x14ac:dyDescent="0.3">
       <c r="A619" t="s">
-        <v>845</v>
+        <v>844</v>
       </c>
     </row>
     <row r="620" spans="1:1" x14ac:dyDescent="0.3">
       <c r="A620" t="s">
-        <v>846</v>
+        <v>845</v>
       </c>
     </row>
     <row r="621" spans="1:1" x14ac:dyDescent="0.3">
@@ -7877,22 +7883,22 @@
     </row>
     <row r="624" spans="1:1" x14ac:dyDescent="0.3">
       <c r="A624" t="s">
-        <v>847</v>
+        <v>846</v>
       </c>
     </row>
     <row r="625" spans="1:1" x14ac:dyDescent="0.3">
       <c r="A625" t="s">
-        <v>848</v>
+        <v>847</v>
       </c>
     </row>
     <row r="626" spans="1:1" x14ac:dyDescent="0.3">
       <c r="A626" t="s">
-        <v>849</v>
+        <v>848</v>
       </c>
     </row>
     <row r="627" spans="1:1" x14ac:dyDescent="0.3">
       <c r="A627" t="s">
-        <v>850</v>
+        <v>849</v>
       </c>
     </row>
     <row r="628" spans="1:1" x14ac:dyDescent="0.3">
@@ -7902,22 +7908,22 @@
     </row>
     <row r="629" spans="1:1" x14ac:dyDescent="0.3">
       <c r="A629" t="s">
-        <v>842</v>
+        <v>841</v>
       </c>
     </row>
     <row r="630" spans="1:1" x14ac:dyDescent="0.3">
       <c r="A630" t="s">
-        <v>843</v>
+        <v>842</v>
       </c>
     </row>
     <row r="631" spans="1:1" x14ac:dyDescent="0.3">
       <c r="A631" t="s">
-        <v>851</v>
+        <v>850</v>
       </c>
     </row>
     <row r="632" spans="1:1" x14ac:dyDescent="0.3">
       <c r="A632" t="s">
-        <v>852</v>
+        <v>851</v>
       </c>
     </row>
     <row r="633" spans="1:1" x14ac:dyDescent="0.3">
@@ -7932,12 +7938,12 @@
     </row>
     <row r="635" spans="1:1" x14ac:dyDescent="0.3">
       <c r="A635" t="s">
-        <v>853</v>
+        <v>852</v>
       </c>
     </row>
     <row r="636" spans="1:1" x14ac:dyDescent="0.3">
       <c r="A636" t="s">
-        <v>711</v>
+        <v>710</v>
       </c>
     </row>
     <row r="637" spans="1:1" x14ac:dyDescent="0.3">
@@ -7957,22 +7963,22 @@
     </row>
     <row r="640" spans="1:1" x14ac:dyDescent="0.3">
       <c r="A640" t="s">
-        <v>854</v>
+        <v>853</v>
       </c>
     </row>
     <row r="641" spans="1:1" x14ac:dyDescent="0.3">
       <c r="A641" t="s">
-        <v>855</v>
+        <v>854</v>
       </c>
     </row>
     <row r="642" spans="1:1" x14ac:dyDescent="0.3">
       <c r="A642" t="s">
-        <v>856</v>
+        <v>855</v>
       </c>
     </row>
     <row r="643" spans="1:1" x14ac:dyDescent="0.3">
       <c r="A643" t="s">
-        <v>857</v>
+        <v>856</v>
       </c>
     </row>
     <row r="644" spans="1:1" x14ac:dyDescent="0.3">
@@ -7987,22 +7993,22 @@
     </row>
     <row r="646" spans="1:1" x14ac:dyDescent="0.3">
       <c r="A646" t="s">
-        <v>858</v>
+        <v>857</v>
       </c>
     </row>
     <row r="647" spans="1:1" x14ac:dyDescent="0.3">
       <c r="A647" t="s">
-        <v>859</v>
+        <v>858</v>
       </c>
     </row>
     <row r="648" spans="1:1" x14ac:dyDescent="0.3">
       <c r="A648" t="s">
-        <v>860</v>
+        <v>859</v>
       </c>
     </row>
     <row r="649" spans="1:1" x14ac:dyDescent="0.3">
       <c r="A649" t="s">
-        <v>861</v>
+        <v>860</v>
       </c>
     </row>
     <row r="650" spans="1:1" x14ac:dyDescent="0.3">
@@ -8012,7 +8018,7 @@
     </row>
     <row r="651" spans="1:1" x14ac:dyDescent="0.3">
       <c r="A651" t="s">
-        <v>862</v>
+        <v>861</v>
       </c>
     </row>
     <row r="652" spans="1:1" x14ac:dyDescent="0.3">
@@ -8022,7 +8028,7 @@
     </row>
     <row r="653" spans="1:1" x14ac:dyDescent="0.3">
       <c r="A653" t="s">
-        <v>863</v>
+        <v>862</v>
       </c>
     </row>
     <row r="654" spans="1:1" x14ac:dyDescent="0.3">
@@ -8052,37 +8058,37 @@
     </row>
     <row r="659" spans="1:1" x14ac:dyDescent="0.3">
       <c r="A659" t="s">
-        <v>864</v>
+        <v>863</v>
       </c>
     </row>
     <row r="660" spans="1:1" x14ac:dyDescent="0.3">
       <c r="A660" t="s">
-        <v>865</v>
+        <v>864</v>
       </c>
     </row>
     <row r="661" spans="1:1" x14ac:dyDescent="0.3">
       <c r="A661" t="s">
-        <v>866</v>
+        <v>865</v>
       </c>
     </row>
     <row r="662" spans="1:1" x14ac:dyDescent="0.3">
       <c r="A662" t="s">
-        <v>867</v>
+        <v>866</v>
       </c>
     </row>
     <row r="663" spans="1:1" x14ac:dyDescent="0.3">
       <c r="A663" t="s">
-        <v>868</v>
+        <v>867</v>
       </c>
     </row>
     <row r="664" spans="1:1" x14ac:dyDescent="0.3">
       <c r="A664" t="s">
-        <v>869</v>
+        <v>868</v>
       </c>
     </row>
     <row r="665" spans="1:1" x14ac:dyDescent="0.3">
       <c r="A665" t="s">
-        <v>870</v>
+        <v>869</v>
       </c>
     </row>
     <row r="666" spans="1:1" x14ac:dyDescent="0.3">
@@ -8097,7 +8103,7 @@
     </row>
     <row r="668" spans="1:1" x14ac:dyDescent="0.3">
       <c r="A668" t="s">
-        <v>871</v>
+        <v>870</v>
       </c>
     </row>
     <row r="669" spans="1:1" x14ac:dyDescent="0.3">
@@ -8107,7 +8113,7 @@
     </row>
     <row r="670" spans="1:1" x14ac:dyDescent="0.3">
       <c r="A670" t="s">
-        <v>872</v>
+        <v>871</v>
       </c>
     </row>
     <row r="671" spans="1:1" x14ac:dyDescent="0.3">
@@ -8122,32 +8128,32 @@
     </row>
     <row r="673" spans="1:1" x14ac:dyDescent="0.3">
       <c r="A673" t="s">
-        <v>873</v>
+        <v>872</v>
       </c>
     </row>
     <row r="674" spans="1:1" x14ac:dyDescent="0.3">
       <c r="A674" t="s">
-        <v>874</v>
+        <v>873</v>
       </c>
     </row>
     <row r="675" spans="1:1" x14ac:dyDescent="0.3">
       <c r="A675" t="s">
-        <v>875</v>
+        <v>874</v>
       </c>
     </row>
     <row r="676" spans="1:1" x14ac:dyDescent="0.3">
       <c r="A676" t="s">
-        <v>876</v>
+        <v>875</v>
       </c>
     </row>
     <row r="677" spans="1:1" x14ac:dyDescent="0.3">
       <c r="A677" t="s">
-        <v>877</v>
+        <v>876</v>
       </c>
     </row>
     <row r="678" spans="1:1" x14ac:dyDescent="0.3">
       <c r="A678" t="s">
-        <v>878</v>
+        <v>877</v>
       </c>
     </row>
     <row r="679" spans="1:1" x14ac:dyDescent="0.3">
@@ -8172,17 +8178,17 @@
     </row>
     <row r="683" spans="1:1" x14ac:dyDescent="0.3">
       <c r="A683" t="s">
-        <v>879</v>
+        <v>878</v>
       </c>
     </row>
     <row r="684" spans="1:1" x14ac:dyDescent="0.3">
       <c r="A684" t="s">
-        <v>880</v>
+        <v>879</v>
       </c>
     </row>
     <row r="685" spans="1:1" x14ac:dyDescent="0.3">
       <c r="A685" t="s">
-        <v>881</v>
+        <v>880</v>
       </c>
     </row>
     <row r="686" spans="1:1" x14ac:dyDescent="0.3">
@@ -8202,7 +8208,7 @@
     </row>
     <row r="689" spans="1:1" x14ac:dyDescent="0.3">
       <c r="A689" t="s">
-        <v>882</v>
+        <v>881</v>
       </c>
     </row>
     <row r="690" spans="1:1" x14ac:dyDescent="0.3">
@@ -8212,27 +8218,27 @@
     </row>
     <row r="691" spans="1:1" x14ac:dyDescent="0.3">
       <c r="A691" t="s">
-        <v>883</v>
+        <v>882</v>
       </c>
     </row>
     <row r="692" spans="1:1" x14ac:dyDescent="0.3">
       <c r="A692" t="s">
-        <v>884</v>
+        <v>883</v>
       </c>
     </row>
     <row r="693" spans="1:1" x14ac:dyDescent="0.3">
       <c r="A693" t="s">
-        <v>885</v>
+        <v>884</v>
       </c>
     </row>
     <row r="694" spans="1:1" x14ac:dyDescent="0.3">
       <c r="A694" t="s">
-        <v>886</v>
+        <v>885</v>
       </c>
     </row>
     <row r="695" spans="1:1" x14ac:dyDescent="0.3">
       <c r="A695" t="s">
-        <v>887</v>
+        <v>886</v>
       </c>
     </row>
     <row r="696" spans="1:1" x14ac:dyDescent="0.3">
@@ -8262,7 +8268,7 @@
     </row>
     <row r="701" spans="1:1" x14ac:dyDescent="0.3">
       <c r="A701" t="s">
-        <v>888</v>
+        <v>887</v>
       </c>
     </row>
     <row r="702" spans="1:1" x14ac:dyDescent="0.3">
@@ -8272,12 +8278,12 @@
     </row>
     <row r="703" spans="1:1" x14ac:dyDescent="0.3">
       <c r="A703" t="s">
-        <v>889</v>
+        <v>888</v>
       </c>
     </row>
     <row r="704" spans="1:1" x14ac:dyDescent="0.3">
       <c r="A704" t="s">
-        <v>669</v>
+        <v>668</v>
       </c>
     </row>
     <row r="705" spans="1:1" x14ac:dyDescent="0.3">
@@ -8292,7 +8298,7 @@
     </row>
     <row r="707" spans="1:1" x14ac:dyDescent="0.3">
       <c r="A707" t="s">
-        <v>890</v>
+        <v>889</v>
       </c>
     </row>
     <row r="708" spans="1:1" x14ac:dyDescent="0.3">
@@ -8322,7 +8328,7 @@
     </row>
     <row r="713" spans="1:1" x14ac:dyDescent="0.3">
       <c r="A713" t="s">
-        <v>891</v>
+        <v>890</v>
       </c>
     </row>
     <row r="714" spans="1:1" x14ac:dyDescent="0.3">
@@ -8342,17 +8348,17 @@
     </row>
     <row r="717" spans="1:1" x14ac:dyDescent="0.3">
       <c r="A717" t="s">
-        <v>669</v>
+        <v>668</v>
       </c>
     </row>
     <row r="718" spans="1:1" x14ac:dyDescent="0.3">
       <c r="A718" t="s">
-        <v>892</v>
+        <v>891</v>
       </c>
     </row>
     <row r="719" spans="1:1" x14ac:dyDescent="0.3">
       <c r="A719" t="s">
-        <v>893</v>
+        <v>892</v>
       </c>
     </row>
     <row r="720" spans="1:1" x14ac:dyDescent="0.3">
@@ -8372,7 +8378,7 @@
     </row>
     <row r="723" spans="1:1" x14ac:dyDescent="0.3">
       <c r="A723" t="s">
-        <v>894</v>
+        <v>893</v>
       </c>
     </row>
     <row r="724" spans="1:1" x14ac:dyDescent="0.3">
@@ -8382,7 +8388,7 @@
     </row>
     <row r="725" spans="1:1" x14ac:dyDescent="0.3">
       <c r="A725" t="s">
-        <v>895</v>
+        <v>894</v>
       </c>
     </row>
     <row r="726" spans="1:1" x14ac:dyDescent="0.3">
@@ -8392,7 +8398,7 @@
     </row>
     <row r="727" spans="1:1" x14ac:dyDescent="0.3">
       <c r="A727" t="s">
-        <v>896</v>
+        <v>895</v>
       </c>
     </row>
     <row r="728" spans="1:1" x14ac:dyDescent="0.3">
@@ -8402,22 +8408,22 @@
     </row>
     <row r="729" spans="1:1" x14ac:dyDescent="0.3">
       <c r="A729" t="s">
-        <v>897</v>
+        <v>896</v>
       </c>
     </row>
     <row r="730" spans="1:1" x14ac:dyDescent="0.3">
       <c r="A730" t="s">
-        <v>898</v>
+        <v>897</v>
       </c>
     </row>
     <row r="731" spans="1:1" x14ac:dyDescent="0.3">
       <c r="A731" t="s">
-        <v>899</v>
+        <v>898</v>
       </c>
     </row>
     <row r="732" spans="1:1" x14ac:dyDescent="0.3">
       <c r="A732" t="s">
-        <v>900</v>
+        <v>899</v>
       </c>
     </row>
     <row r="733" spans="1:1" x14ac:dyDescent="0.3">
@@ -8437,7 +8443,7 @@
     </row>
     <row r="736" spans="1:1" x14ac:dyDescent="0.3">
       <c r="A736" t="s">
-        <v>901</v>
+        <v>900</v>
       </c>
     </row>
     <row r="737" spans="1:1" x14ac:dyDescent="0.3">
@@ -8457,7 +8463,7 @@
     </row>
     <row r="740" spans="1:1" x14ac:dyDescent="0.3">
       <c r="A740" t="s">
-        <v>902</v>
+        <v>901</v>
       </c>
     </row>
     <row r="741" spans="1:1" x14ac:dyDescent="0.3">
@@ -8467,7 +8473,7 @@
     </row>
     <row r="742" spans="1:1" x14ac:dyDescent="0.3">
       <c r="A742" t="s">
-        <v>903</v>
+        <v>902</v>
       </c>
     </row>
     <row r="743" spans="1:1" x14ac:dyDescent="0.3">
@@ -8482,12 +8488,12 @@
     </row>
     <row r="745" spans="1:1" x14ac:dyDescent="0.3">
       <c r="A745" t="s">
-        <v>904</v>
+        <v>903</v>
       </c>
     </row>
     <row r="746" spans="1:1" x14ac:dyDescent="0.3">
       <c r="A746" t="s">
-        <v>905</v>
+        <v>904</v>
       </c>
     </row>
     <row r="747" spans="1:1" x14ac:dyDescent="0.3">
@@ -8507,7 +8513,7 @@
     </row>
     <row r="750" spans="1:1" x14ac:dyDescent="0.3">
       <c r="A750" t="s">
-        <v>906</v>
+        <v>905</v>
       </c>
     </row>
     <row r="751" spans="1:1" x14ac:dyDescent="0.3">
@@ -8542,7 +8548,7 @@
     </row>
     <row r="757" spans="1:1" x14ac:dyDescent="0.3">
       <c r="A757" t="s">
-        <v>907</v>
+        <v>906</v>
       </c>
     </row>
     <row r="758" spans="1:1" x14ac:dyDescent="0.3">
@@ -8572,7 +8578,7 @@
     </row>
     <row r="763" spans="1:1" x14ac:dyDescent="0.3">
       <c r="A763" t="s">
-        <v>908</v>
+        <v>907</v>
       </c>
     </row>
     <row r="764" spans="1:1" x14ac:dyDescent="0.3">
@@ -8597,12 +8603,12 @@
     </row>
     <row r="768" spans="1:1" x14ac:dyDescent="0.3">
       <c r="A768" t="s">
-        <v>909</v>
+        <v>908</v>
       </c>
     </row>
     <row r="769" spans="1:1" x14ac:dyDescent="0.3">
       <c r="A769" t="s">
-        <v>669</v>
+        <v>668</v>
       </c>
     </row>
     <row r="770" spans="1:1" x14ac:dyDescent="0.3">
@@ -8612,7 +8618,7 @@
     </row>
     <row r="771" spans="1:1" x14ac:dyDescent="0.3">
       <c r="A771" t="s">
-        <v>910</v>
+        <v>909</v>
       </c>
     </row>
     <row r="772" spans="1:1" x14ac:dyDescent="0.3">
@@ -8632,22 +8638,22 @@
     </row>
     <row r="775" spans="1:1" x14ac:dyDescent="0.3">
       <c r="A775" t="s">
-        <v>911</v>
+        <v>910</v>
       </c>
     </row>
     <row r="776" spans="1:1" x14ac:dyDescent="0.3">
       <c r="A776" t="s">
-        <v>669</v>
+        <v>668</v>
       </c>
     </row>
     <row r="777" spans="1:1" x14ac:dyDescent="0.3">
       <c r="A777" t="s">
-        <v>912</v>
+        <v>911</v>
       </c>
     </row>
     <row r="778" spans="1:1" x14ac:dyDescent="0.3">
       <c r="A778" t="s">
-        <v>913</v>
+        <v>912</v>
       </c>
     </row>
     <row r="779" spans="1:1" x14ac:dyDescent="0.3">
@@ -8657,27 +8663,27 @@
     </row>
     <row r="780" spans="1:1" x14ac:dyDescent="0.3">
       <c r="A780" t="s">
-        <v>914</v>
+        <v>913</v>
       </c>
     </row>
     <row r="781" spans="1:1" x14ac:dyDescent="0.3">
       <c r="A781" t="s">
-        <v>915</v>
+        <v>914</v>
       </c>
     </row>
     <row r="782" spans="1:1" x14ac:dyDescent="0.3">
       <c r="A782" t="s">
-        <v>916</v>
+        <v>915</v>
       </c>
     </row>
     <row r="783" spans="1:1" x14ac:dyDescent="0.3">
       <c r="A783" t="s">
-        <v>917</v>
+        <v>916</v>
       </c>
     </row>
     <row r="784" spans="1:1" x14ac:dyDescent="0.3">
       <c r="A784" t="s">
-        <v>918</v>
+        <v>917</v>
       </c>
     </row>
     <row r="785" spans="1:1" x14ac:dyDescent="0.3">
@@ -8687,17 +8693,17 @@
     </row>
     <row r="786" spans="1:1" x14ac:dyDescent="0.3">
       <c r="A786" t="s">
-        <v>919</v>
+        <v>918</v>
       </c>
     </row>
     <row r="787" spans="1:1" x14ac:dyDescent="0.3">
       <c r="A787" t="s">
-        <v>920</v>
+        <v>919</v>
       </c>
     </row>
     <row r="788" spans="1:1" x14ac:dyDescent="0.3">
       <c r="A788" t="s">
-        <v>921</v>
+        <v>920</v>
       </c>
     </row>
     <row r="789" spans="1:1" x14ac:dyDescent="0.3">
@@ -8712,7 +8718,7 @@
     </row>
     <row r="791" spans="1:1" x14ac:dyDescent="0.3">
       <c r="A791" t="s">
-        <v>922</v>
+        <v>921</v>
       </c>
     </row>
     <row r="792" spans="1:1" x14ac:dyDescent="0.3">
@@ -8722,37 +8728,37 @@
     </row>
     <row r="793" spans="1:1" x14ac:dyDescent="0.3">
       <c r="A793" t="s">
-        <v>923</v>
+        <v>922</v>
       </c>
     </row>
     <row r="794" spans="1:1" x14ac:dyDescent="0.3">
       <c r="A794" t="s">
-        <v>924</v>
+        <v>923</v>
       </c>
     </row>
     <row r="795" spans="1:1" x14ac:dyDescent="0.3">
       <c r="A795" t="s">
-        <v>925</v>
+        <v>924</v>
       </c>
     </row>
     <row r="796" spans="1:1" x14ac:dyDescent="0.3">
       <c r="A796" t="s">
-        <v>926</v>
+        <v>925</v>
       </c>
     </row>
     <row r="797" spans="1:1" x14ac:dyDescent="0.3">
       <c r="A797" t="s">
-        <v>927</v>
+        <v>926</v>
       </c>
     </row>
     <row r="798" spans="1:1" x14ac:dyDescent="0.3">
       <c r="A798" t="s">
-        <v>928</v>
+        <v>927</v>
       </c>
     </row>
     <row r="799" spans="1:1" x14ac:dyDescent="0.3">
       <c r="A799" t="s">
-        <v>928</v>
+        <v>927</v>
       </c>
     </row>
     <row r="800" spans="1:1" x14ac:dyDescent="0.3">
@@ -8767,7 +8773,7 @@
     </row>
     <row r="802" spans="1:1" x14ac:dyDescent="0.3">
       <c r="A802" t="s">
-        <v>606</v>
+        <v>605</v>
       </c>
     </row>
     <row r="803" spans="1:1" x14ac:dyDescent="0.3">
@@ -8777,7 +8783,7 @@
     </row>
     <row r="804" spans="1:1" x14ac:dyDescent="0.3">
       <c r="A804" t="s">
-        <v>669</v>
+        <v>668</v>
       </c>
     </row>
     <row r="805" spans="1:1" x14ac:dyDescent="0.3">
@@ -8797,7 +8803,7 @@
     </row>
     <row r="808" spans="1:1" x14ac:dyDescent="0.3">
       <c r="A808" t="s">
-        <v>669</v>
+        <v>668</v>
       </c>
     </row>
     <row r="809" spans="1:1" x14ac:dyDescent="0.3">
@@ -8807,7 +8813,7 @@
     </row>
     <row r="810" spans="1:1" x14ac:dyDescent="0.3">
       <c r="A810" t="s">
-        <v>669</v>
+        <v>668</v>
       </c>
     </row>
     <row r="811" spans="1:1" x14ac:dyDescent="0.3">
@@ -8857,12 +8863,12 @@
     </row>
     <row r="820" spans="1:1" x14ac:dyDescent="0.3">
       <c r="A820" t="s">
-        <v>929</v>
+        <v>928</v>
       </c>
     </row>
     <row r="821" spans="1:1" x14ac:dyDescent="0.3">
       <c r="A821" t="s">
-        <v>930</v>
+        <v>929</v>
       </c>
     </row>
     <row r="822" spans="1:1" x14ac:dyDescent="0.3">
@@ -8872,17 +8878,17 @@
     </row>
     <row r="823" spans="1:1" x14ac:dyDescent="0.3">
       <c r="A823" t="s">
-        <v>931</v>
+        <v>930</v>
       </c>
     </row>
     <row r="824" spans="1:1" x14ac:dyDescent="0.3">
       <c r="A824" t="s">
-        <v>932</v>
+        <v>931</v>
       </c>
     </row>
     <row r="825" spans="1:1" x14ac:dyDescent="0.3">
       <c r="A825" t="s">
-        <v>933</v>
+        <v>932</v>
       </c>
     </row>
     <row r="826" spans="1:1" x14ac:dyDescent="0.3">
@@ -8907,7 +8913,7 @@
     </row>
     <row r="830" spans="1:1" x14ac:dyDescent="0.3">
       <c r="A830" t="s">
-        <v>934</v>
+        <v>933</v>
       </c>
     </row>
     <row r="831" spans="1:1" x14ac:dyDescent="0.3">
@@ -8922,22 +8928,22 @@
     </row>
     <row r="833" spans="1:1" x14ac:dyDescent="0.3">
       <c r="A833" t="s">
-        <v>935</v>
+        <v>934</v>
       </c>
     </row>
     <row r="834" spans="1:1" x14ac:dyDescent="0.3">
       <c r="A834" t="s">
-        <v>936</v>
+        <v>935</v>
       </c>
     </row>
     <row r="835" spans="1:1" x14ac:dyDescent="0.3">
       <c r="A835" t="s">
-        <v>937</v>
+        <v>936</v>
       </c>
     </row>
     <row r="836" spans="1:1" x14ac:dyDescent="0.3">
       <c r="A836" t="s">
-        <v>938</v>
+        <v>937</v>
       </c>
     </row>
     <row r="837" spans="1:1" x14ac:dyDescent="0.3">
@@ -8947,12 +8953,12 @@
     </row>
     <row r="838" spans="1:1" x14ac:dyDescent="0.3">
       <c r="A838" t="s">
-        <v>939</v>
+        <v>938</v>
       </c>
     </row>
     <row r="839" spans="1:1" x14ac:dyDescent="0.3">
       <c r="A839" t="s">
-        <v>940</v>
+        <v>939</v>
       </c>
     </row>
     <row r="840" spans="1:1" x14ac:dyDescent="0.3">
@@ -8962,12 +8968,12 @@
     </row>
     <row r="841" spans="1:1" x14ac:dyDescent="0.3">
       <c r="A841" t="s">
-        <v>941</v>
+        <v>940</v>
       </c>
     </row>
     <row r="842" spans="1:1" x14ac:dyDescent="0.3">
       <c r="A842" t="s">
-        <v>942</v>
+        <v>941</v>
       </c>
     </row>
     <row r="843" spans="1:1" x14ac:dyDescent="0.3">
@@ -8977,12 +8983,12 @@
     </row>
     <row r="844" spans="1:1" x14ac:dyDescent="0.3">
       <c r="A844" t="s">
-        <v>943</v>
+        <v>942</v>
       </c>
     </row>
     <row r="845" spans="1:1" x14ac:dyDescent="0.3">
       <c r="A845" t="s">
-        <v>944</v>
+        <v>943</v>
       </c>
     </row>
     <row r="846" spans="1:1" x14ac:dyDescent="0.3">
@@ -8997,7 +9003,7 @@
     </row>
     <row r="848" spans="1:1" x14ac:dyDescent="0.3">
       <c r="A848" t="s">
-        <v>945</v>
+        <v>944</v>
       </c>
     </row>
     <row r="849" spans="1:1" x14ac:dyDescent="0.3">
@@ -9022,7 +9028,7 @@
     </row>
     <row r="853" spans="1:1" x14ac:dyDescent="0.3">
       <c r="A853" t="s">
-        <v>946</v>
+        <v>945</v>
       </c>
     </row>
     <row r="854" spans="1:1" x14ac:dyDescent="0.3">
@@ -9037,17 +9043,17 @@
     </row>
     <row r="856" spans="1:1" x14ac:dyDescent="0.3">
       <c r="A856" t="s">
-        <v>947</v>
+        <v>946</v>
       </c>
     </row>
     <row r="857" spans="1:1" x14ac:dyDescent="0.3">
       <c r="A857" t="s">
-        <v>948</v>
+        <v>947</v>
       </c>
     </row>
     <row r="858" spans="1:1" x14ac:dyDescent="0.3">
       <c r="A858" t="s">
-        <v>949</v>
+        <v>948</v>
       </c>
     </row>
     <row r="859" spans="1:1" x14ac:dyDescent="0.3">
@@ -9062,27 +9068,27 @@
     </row>
     <row r="861" spans="1:1" x14ac:dyDescent="0.3">
       <c r="A861" t="s">
-        <v>950</v>
+        <v>949</v>
       </c>
     </row>
     <row r="862" spans="1:1" x14ac:dyDescent="0.3">
       <c r="A862" t="s">
-        <v>951</v>
+        <v>950</v>
       </c>
     </row>
     <row r="863" spans="1:1" x14ac:dyDescent="0.3">
       <c r="A863" t="s">
-        <v>952</v>
+        <v>951</v>
       </c>
     </row>
     <row r="864" spans="1:1" x14ac:dyDescent="0.3">
       <c r="A864" t="s">
-        <v>953</v>
+        <v>952</v>
       </c>
     </row>
     <row r="865" spans="1:1" x14ac:dyDescent="0.3">
       <c r="A865" t="s">
-        <v>954</v>
+        <v>953</v>
       </c>
     </row>
     <row r="866" spans="1:1" x14ac:dyDescent="0.3">
@@ -9097,17 +9103,17 @@
     </row>
     <row r="868" spans="1:1" x14ac:dyDescent="0.3">
       <c r="A868" t="s">
-        <v>955</v>
+        <v>954</v>
       </c>
     </row>
     <row r="869" spans="1:1" x14ac:dyDescent="0.3">
       <c r="A869" t="s">
-        <v>956</v>
+        <v>955</v>
       </c>
     </row>
     <row r="870" spans="1:1" x14ac:dyDescent="0.3">
       <c r="A870" t="s">
-        <v>957</v>
+        <v>956</v>
       </c>
     </row>
     <row r="871" spans="1:1" x14ac:dyDescent="0.3">
@@ -9142,7 +9148,7 @@
     </row>
     <row r="877" spans="1:1" x14ac:dyDescent="0.3">
       <c r="A877" t="s">
-        <v>958</v>
+        <v>957</v>
       </c>
     </row>
     <row r="878" spans="1:1" x14ac:dyDescent="0.3">
@@ -9152,7 +9158,7 @@
     </row>
     <row r="879" spans="1:1" x14ac:dyDescent="0.3">
       <c r="A879" t="s">
-        <v>959</v>
+        <v>958</v>
       </c>
     </row>
     <row r="880" spans="1:1" x14ac:dyDescent="0.3">
@@ -9167,7 +9173,7 @@
     </row>
     <row r="882" spans="1:1" x14ac:dyDescent="0.3">
       <c r="A882" t="s">
-        <v>960</v>
+        <v>959</v>
       </c>
     </row>
     <row r="883" spans="1:1" x14ac:dyDescent="0.3">
@@ -9192,7 +9198,7 @@
     </row>
     <row r="887" spans="1:1" x14ac:dyDescent="0.3">
       <c r="A887" t="s">
-        <v>961</v>
+        <v>960</v>
       </c>
     </row>
     <row r="888" spans="1:1" x14ac:dyDescent="0.3">
@@ -9202,12 +9208,12 @@
     </row>
     <row r="889" spans="1:1" x14ac:dyDescent="0.3">
       <c r="A889" t="s">
-        <v>962</v>
+        <v>961</v>
       </c>
     </row>
     <row r="890" spans="1:1" x14ac:dyDescent="0.3">
       <c r="A890" t="s">
-        <v>963</v>
+        <v>962</v>
       </c>
     </row>
     <row r="891" spans="1:1" x14ac:dyDescent="0.3">
@@ -9227,7 +9233,7 @@
     </row>
     <row r="894" spans="1:1" x14ac:dyDescent="0.3">
       <c r="A894" t="s">
-        <v>964</v>
+        <v>963</v>
       </c>
     </row>
     <row r="895" spans="1:1" x14ac:dyDescent="0.3">
@@ -9252,7 +9258,7 @@
     </row>
     <row r="899" spans="1:1" x14ac:dyDescent="0.3">
       <c r="A899" t="s">
-        <v>965</v>
+        <v>964</v>
       </c>
     </row>
     <row r="900" spans="1:1" x14ac:dyDescent="0.3">
@@ -9272,17 +9278,17 @@
     </row>
     <row r="903" spans="1:1" x14ac:dyDescent="0.3">
       <c r="A903" t="s">
-        <v>947</v>
+        <v>946</v>
       </c>
     </row>
     <row r="904" spans="1:1" x14ac:dyDescent="0.3">
       <c r="A904" t="s">
-        <v>966</v>
+        <v>965</v>
       </c>
     </row>
     <row r="905" spans="1:1" x14ac:dyDescent="0.3">
       <c r="A905" t="s">
-        <v>967</v>
+        <v>966</v>
       </c>
     </row>
     <row r="906" spans="1:1" x14ac:dyDescent="0.3">
@@ -9302,7 +9308,7 @@
     </row>
     <row r="909" spans="1:1" x14ac:dyDescent="0.3">
       <c r="A909" t="s">
-        <v>968</v>
+        <v>967</v>
       </c>
     </row>
     <row r="910" spans="1:1" x14ac:dyDescent="0.3">
@@ -9317,17 +9323,17 @@
     </row>
     <row r="912" spans="1:1" x14ac:dyDescent="0.3">
       <c r="A912" t="s">
-        <v>969</v>
+        <v>968</v>
       </c>
     </row>
     <row r="913" spans="1:1" x14ac:dyDescent="0.3">
       <c r="A913" t="s">
-        <v>970</v>
+        <v>969</v>
       </c>
     </row>
     <row r="914" spans="1:1" x14ac:dyDescent="0.3">
       <c r="A914" t="s">
-        <v>971</v>
+        <v>970</v>
       </c>
     </row>
     <row r="915" spans="1:1" x14ac:dyDescent="0.3">
@@ -9387,12 +9393,12 @@
     </row>
     <row r="926" spans="1:1" x14ac:dyDescent="0.3">
       <c r="A926" t="s">
-        <v>972</v>
+        <v>971</v>
       </c>
     </row>
     <row r="927" spans="1:1" x14ac:dyDescent="0.3">
       <c r="A927" t="s">
-        <v>973</v>
+        <v>972</v>
       </c>
     </row>
     <row r="928" spans="1:1" x14ac:dyDescent="0.3">
@@ -9417,7 +9423,7 @@
     </row>
     <row r="932" spans="1:1" x14ac:dyDescent="0.3">
       <c r="A932" t="s">
-        <v>974</v>
+        <v>973</v>
       </c>
     </row>
     <row r="933" spans="1:1" x14ac:dyDescent="0.3">
@@ -9442,7 +9448,7 @@
     </row>
     <row r="937" spans="1:1" x14ac:dyDescent="0.3">
       <c r="A937" t="s">
-        <v>975</v>
+        <v>974</v>
       </c>
     </row>
     <row r="938" spans="1:1" x14ac:dyDescent="0.3">
@@ -9462,7 +9468,7 @@
     </row>
     <row r="941" spans="1:1" x14ac:dyDescent="0.3">
       <c r="A941" t="s">
-        <v>976</v>
+        <v>975</v>
       </c>
     </row>
     <row r="942" spans="1:1" x14ac:dyDescent="0.3">
@@ -9492,7 +9498,7 @@
     </row>
     <row r="947" spans="1:1" x14ac:dyDescent="0.3">
       <c r="A947" t="s">
-        <v>977</v>
+        <v>976</v>
       </c>
     </row>
     <row r="948" spans="1:1" x14ac:dyDescent="0.3">
@@ -9507,7 +9513,7 @@
     </row>
     <row r="950" spans="1:1" x14ac:dyDescent="0.3">
       <c r="A950" t="s">
-        <v>978</v>
+        <v>977</v>
       </c>
     </row>
     <row r="951" spans="1:1" x14ac:dyDescent="0.3">
@@ -9537,7 +9543,7 @@
     </row>
     <row r="956" spans="1:1" x14ac:dyDescent="0.3">
       <c r="A956" t="s">
-        <v>979</v>
+        <v>978</v>
       </c>
     </row>
     <row r="957" spans="1:1" x14ac:dyDescent="0.3">
@@ -9547,7 +9553,7 @@
     </row>
     <row r="958" spans="1:1" x14ac:dyDescent="0.3">
       <c r="A958" t="s">
-        <v>980</v>
+        <v>979</v>
       </c>
     </row>
     <row r="959" spans="1:1" x14ac:dyDescent="0.3">
@@ -9557,7 +9563,7 @@
     </row>
     <row r="960" spans="1:1" x14ac:dyDescent="0.3">
       <c r="A960" t="s">
-        <v>981</v>
+        <v>980</v>
       </c>
     </row>
     <row r="961" spans="1:1" x14ac:dyDescent="0.3">
@@ -9572,12 +9578,12 @@
     </row>
     <row r="963" spans="1:1" x14ac:dyDescent="0.3">
       <c r="A963" t="s">
-        <v>982</v>
+        <v>981</v>
       </c>
     </row>
     <row r="964" spans="1:1" x14ac:dyDescent="0.3">
       <c r="A964" t="s">
-        <v>983</v>
+        <v>982</v>
       </c>
     </row>
     <row r="965" spans="1:1" x14ac:dyDescent="0.3">
@@ -9602,7 +9608,7 @@
     </row>
     <row r="969" spans="1:1" x14ac:dyDescent="0.3">
       <c r="A969" t="s">
-        <v>984</v>
+        <v>983</v>
       </c>
     </row>
     <row r="970" spans="1:1" x14ac:dyDescent="0.3">
@@ -9617,7 +9623,7 @@
     </row>
     <row r="972" spans="1:1" x14ac:dyDescent="0.3">
       <c r="A972" t="s">
-        <v>985</v>
+        <v>984</v>
       </c>
     </row>
     <row r="973" spans="1:1" x14ac:dyDescent="0.3">
@@ -9677,7 +9683,7 @@
     </row>
     <row r="984" spans="1:1" x14ac:dyDescent="0.3">
       <c r="A984" t="s">
-        <v>986</v>
+        <v>985</v>
       </c>
     </row>
     <row r="985" spans="1:1" x14ac:dyDescent="0.3">
@@ -9697,7 +9703,7 @@
     </row>
     <row r="988" spans="1:1" x14ac:dyDescent="0.3">
       <c r="A988" t="s">
-        <v>987</v>
+        <v>986</v>
       </c>
     </row>
     <row r="989" spans="1:1" x14ac:dyDescent="0.3">
@@ -9747,7 +9753,7 @@
     </row>
     <row r="998" spans="1:1" x14ac:dyDescent="0.3">
       <c r="A998" t="s">
-        <v>988</v>
+        <v>987</v>
       </c>
     </row>
     <row r="999" spans="1:1" x14ac:dyDescent="0.3">

</xml_diff>